<commit_message>
Rebuild profiles on an M&A-first axis; add 5 fintech M&A shops
- New columns: FinTech Coverage (dedicated / named group / within FIG /
  none) and Crypto M&A Credits (count), so the sheet sorts on M&A depth
- ECM/DAT and Restructuring columns relabelled as context-only
- Added Piper Sandler, William Blair, Raymond James, D.A. Davidson
  (ex-Marlin team) and Arma Partners - fintech M&A shops the
  crypto-deal-sourced list systematically missed
- 39 firms total

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WXzZsq4Qrn4tV9mBn34Mo
</commit_message>
<xml_diff>
--- a/IB_Target_Profiles.xlsx
+++ b/IB_Target_Profiles.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Profiles" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bank Profiles'!$A$5:$I$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bank Profiles'!$A$5:$K$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,13 +103,16 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -480,18 +483,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -504,7 +509,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Target-group precision for the crypto/fintech M&amp;A and ECM lane  |  Restructuring credits shown separately as context only  |  CBS Class of 2028, summer 2027 associate cycle</t>
+          <t>M&amp;A-FIRST view: target-group precision for the crypto/fintech M&amp;A lane  |  ECM and restructuring credits shown separately as CONTEXT ONLY  |  CBS Class of 2028, summer 2027 associate cycle</t>
         </is>
       </c>
     </row>
@@ -529,35 +534,45 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>FinTech Coverage</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>Group / Department to Target</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Department Notes &amp; Traps</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Crypto M&amp;A Credits</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Crypto &amp; Fintech M&amp;A Mandates</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>ECM / DAT / Capital Markets</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Restructuring (context only — not your target)</t>
-        </is>
-      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
+          <t>ECM / DAT / Capital Markets (context — not your target)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Restructuring (context — not your target)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
           <t>CBS Alumni Contact</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
@@ -576,31 +591,41 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
           <t>Global Banking &amp; Markets - Financial Institutions Group (FIG); fintech coverage sits in FIG/TMT. Separate Digital Assets team in GBM.</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Largest crypto M&amp;A count in the dataset, but crypto is a subset of a vast platform - you are recruiting into FIG, not into a crypto desk.</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>GTreasury $1B (excl. sell-side for Hg, Oct 2025); Core Scientific / CoreWeave $9B (buy-side, Jul 2025); Equiniti $4.2B (excl. buy-side for Bullish, May 2026); Reap up to $600M (co-sell, GS Asia, May 2026)</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Top-tier ECM franchise; crypto IPO wave (Circle CRCL Jun 2025, Bullish, Gemini GEMI Sep 2025) - VERIFY which bookrunner roles GS held. NEOS up to $2.25B was GS as principal buyer (GBM), not an advisory mandate.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="7" t="n"/>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="8" t="n"/>
     </row>
     <row r="7" ht="92" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -615,35 +640,45 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
+          <t>Named: FIG FinTech Coverage</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
           <t>Investment Banking - FIG, FinTech coverage; Technology group adjacent.</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Most active BB in crypto by mandate count. Larger associate class than any EB. Leveraged finance sits alongside - the Long Ridge bridge came from the same relationship.</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Bitstamp $200M (excl. buy-side for Robinhood, Jun 2024); Long Ridge $1.5B (co-buy-side for MARA + bridge loan, Apr 2026); Kiavi $717M (excl. buy-side for Figure/Sixth Street, Jun 2026); NEOS up to $2.25B (excl. sell-side, Aug 2026)</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Long Ridge bridge financing (Apr 2026). Full ECM platform - confirm crypto/fintech issuance roles.</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>Taiwo O. - FIG FinTech Coverage, CBS MBA</t>
         </is>
       </c>
-      <c r="I7" s="7" t="n"/>
+      <c r="K7" s="8" t="n"/>
     </row>
     <row r="8" ht="92" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -658,31 +693,41 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
+          <t>Dedicated FinTech coverage in IB</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
           <t>Investment Banking - FIG / Financial Technology coverage.</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>TRAP: Kinexys (ex-Onyx) is JPM's blockchain PRODUCT unit - deposit tokens, tokenized repo. It is not investment banking and will not lead to an M&amp;A seat. Target FIG.</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Adecoagro ~$615.5M tender (excl. sell-side vs Tether, Mar 2025); WonderFi C$250M (buy-side for Robinhood, May 2025)</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Full ECM platform; reported role in the Circle (CRCL) IPO - VERIFY.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="7" t="n"/>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="n"/>
+      <c r="K8" s="8" t="n"/>
     </row>
     <row r="9" ht="92" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -697,31 +742,41 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
           <t>Banking - FIG / Financial Technology; digital assets coverage within FIG.</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>TRAP: Citi Token Services is a product/treasury build, not IB. Citi's crypto credit is an ECM/DAT one, not M&amp;A.</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Securitize $1.25B pre-money de-SPAC (FA to Securitize + co-placement, Oct 2025; NYSE: SECZ Jul 2026)</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="7" t="n"/>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="8" t="n"/>
     </row>
     <row r="10" ht="92" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -736,35 +791,45 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
+          <t>Named: Head of FinTech &amp; AI</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
           <t>Investment Banking - Global Financial Institutions; FinTech coverage (Head of FinTech &amp; AI sits in London).</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto M&amp;A credit 2024-26. Included for fintech breadth and the E*TRADE crypto build. Verify before pitching crypto here.</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>None disclosed in crypto. (Historic fintech/LatAm depth - Gol/Smiles was alongside MS, which is your own credential.)</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Full ECM platform - verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Richard Pilipuitis - MD, Head of FinTech &amp; AI (CBS exec-ed, not a degree - soft tie)</t>
         </is>
       </c>
-      <c r="I10" s="7" t="n"/>
+      <c r="K10" s="8" t="n"/>
     </row>
     <row r="11" ht="92" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -779,35 +844,45 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
           <t>Investment Banking - Global FIG / FinTech; Technology group adjacent.</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto M&amp;A credit 2024-26. Fintech coverage is real; crypto is not a stated franchise.</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Full ECM platform - verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Yusuf Ibrahim - IB Associate, fintech/tech, CBS MBA '25</t>
         </is>
       </c>
-      <c r="I11" s="7" t="n"/>
+      <c r="K11" s="8" t="n"/>
     </row>
     <row r="12" ht="92" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -822,31 +897,41 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
           <t>Corporate &amp; Investment Banking - FIG / Financial Technology.</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Single syndicate appearance; not a crypto franchise. Low priority unless a relationship appears.</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>1 (syndicate)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Equiniti $4.2B (sell-side syndicate alongside Evercore/FT Partners leads, May 2026)</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="7" t="n"/>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="8" t="n"/>
     </row>
     <row r="13" ht="92" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -861,31 +946,41 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
+          <t>Within FIG (verify if branded)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
           <t>STRATEGIC ADVISORY (M&amp;A). NOT RSSG.</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>CRITICAL: RSSG (Restructuring &amp; Special Situations Group) is a separate, MBA-heavy track and is where the Core Scientific Ch.11 sat - the tracks split early. Park Hill (fund placement) is a third arm. All the Payward M&amp;A work is Strategic Advisory. Say 'strategic advisory' in every conversation.</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>NinjaTrader $1.5B (buy-side for Kraken/Payward, Mar 2025); Core Scientific $9B (co-sell with Moelis, Jul 2025); Bitnomial up to $550M (excl. sell-side, Apr 2026); Reap up to $600M (buy-side for Payward, May 2026)</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Core Scientific Ch.11 debtors (RSSG) - context only</t>
         </is>
       </c>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="8" t="n"/>
     </row>
     <row r="14" ht="92" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -900,31 +995,41 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
           <t>Advisory - FIG / Financial Technology coverage. Capital Markets Advisory (ECM) is a distinct group.</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Largest associate class among the EBs and a consistent CBS hirer. Crypto evidence is thin (one credit) - lead with the fintech franchise, not a crypto thesis.</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Equiniti $4.2B (co-lead sell-side for Siris with FT Partners, May 2026)</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Capital Markets Advisory group; verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="7" t="n"/>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="8" t="n"/>
     </row>
     <row r="15" ht="92" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -939,31 +1044,41 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
           <t>Generalist M&amp;A coverage. Recapitalization &amp; Restructuring (R&amp;R) is the separate arm.</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Its crypto reputation is 60% restructuring (Voyager, Genesis, BlockFi debtors). If you have ruled out Rx, only two of its five credits are relevant - and staffing can cross between M&amp;A and R&amp;R.</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Stronghold Digital $125M (buy-side for Bitfarms, Aug 2024); Core Scientific $9B (co-sell with PJT, Jul 2025)</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Genesis, Voyager, BlockFi debtors - context only</t>
         </is>
       </c>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="7" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="8" t="n"/>
     </row>
     <row r="16" ht="92" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -978,35 +1093,45 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
+          <t>Named: FinTech &amp; Wealth</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
           <t>Investment Banking - FINTECH &amp; WEALTH group (within FIG). Technology group adjacent. Full ECM platform in-house.</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Only firm combining three crypto M&amp;A sell-sides, real ECM, the largest associate class of the group, and a CBS alum leading the exact coverage group.</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>NinjaTrader $1.5B (sell-side, Mar 2025); Long Ridge $1.5B (co-sell with Lazard for FTAI, Apr 2026); Kiavi $717M (sell-side for Figure, Jun 2026)</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Full ECM/leveraged finance platform - the strongest ECM offering of any non-BB on this list. Verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>FTX creditors committee - context only</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>John Erwin - MD, FinTech &amp; Wealth Investment Banking, CBS MBA '06</t>
         </is>
       </c>
-      <c r="I16" s="7" t="n"/>
+      <c r="K16" s="8" t="n"/>
     </row>
     <row r="17" ht="92" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1021,31 +1146,41 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
           <t>Financial Advisory - FIG; the Long Ridge mandate ran through Power &amp; Energy Infrastructure.</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Its single crypto credit was a POWER asset sale, not a crypto business - do not overstate it as a digital-assets franchise.</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>Long Ridge $1.5B (co-sell with Jefferies for FTAI, Apr 2026)</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="7" t="n"/>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="8" t="n"/>
     </row>
     <row r="18" ht="92" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1060,31 +1195,41 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
+          <t>None - generalist staffing</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
           <t>Generalist advisory - no formal industry groups; industry-agnostic staffing.</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>ZERO crypto M&amp;A credits. Its only crypto work is the Celsius Ch.11 debtor role. Smallest class in the market.</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Celsius Ch.11 debtors (~$20.1M fee allocation) - context only</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="8" t="n"/>
     </row>
     <row r="19" ht="92" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1099,31 +1244,41 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
           <t>Single Advisory platform (M&amp;A and restructuring are not separately branded).</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>ZERO crypto M&amp;A credits. Both crypto engagements are restructuring - FTX debtors and Celsius creditors. Its crypto reputation is entirely estates.</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>FTX debtors (ran the LedgerX and FTX Europe sales); Celsius creditors - context only</t>
         </is>
       </c>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="8" t="n"/>
     </row>
     <row r="20" ht="92" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1138,31 +1293,41 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
+          <t>Named: FinTech (Corporate Finance)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
           <t>CORPORATE FINANCE (M&amp;A) - has a real FinTech group. Financial Restructuring is the separate arm where the crypto work sat.</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>ZERO crypto M&amp;A credits; the Genesis role was creditor-side Rx. The Corporate Finance FinTech group is legitimate for fintech M&amp;A - but that is a fintech pitch, not a crypto one.</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>0 crypto / active fintech</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>None in crypto (Corporate Finance FinTech practice is active in payments/specialty finance broadly)</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Genesis creditors - context only</t>
         </is>
       </c>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="8" t="n"/>
     </row>
     <row r="21" ht="92" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1177,31 +1342,41 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
           <t>Investment Banking - FIG / Technology coverage.</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto M&amp;A credits 2024-26 - the weakest evidence of any Tier 1 name. Only worth time if networking comes free.</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="7" t="n"/>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="8" t="n"/>
     </row>
     <row r="22" ht="92" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1216,31 +1391,41 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
+          <t>None - TMT generalist</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
           <t>Generalist merchant bank, TMT &amp; media focus; no dedicated crypto or fintech group.</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Founder-led (Aryeh Bourkoff), very small intake, relationship-driven. The Semler mandate shows real digital-asset appetite but arrived through generalist coverage.</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Semler Scientific ~$1.4B all-stock (EXCLUSIVE sell-side vs Strive, Sep 2025 - the first DAT stock-for-stock merger); Equiniti $4.2B (sell-side syndicate, May 2026)</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="7" t="n"/>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="8" t="n"/>
     </row>
     <row r="23" ht="92" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -1255,35 +1440,45 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
+          <t>ENTIRE FIRM</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
           <t>No traditional department structure - organized in vertical deal teams; the relevant vertical is Blockchain / Digital Assets. Founder-led (Steve McLaughlin).</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>The single purest fintech M&amp;A franchise on this list: 100% fintech, zero restructuring. Hires associates DIRECTLY via Greenhouse (no OCR), so it does not compete with your Sept-Jan calendar. Culture is famously demanding - diligence with former juniors before committing.</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Hidden Road $1.25B (sell-side for Ripple, Apr 2025 - now Ripple Prime); Deribit $2.9B, $3.9-4.3B at close (sell-side for Coinbase, May 2025); WonderFi C$250M (sell-side, May 2025); Equiniti $4.2B (co-lead sell-side with Evercore, May 2026)</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Private capital raising is a core FTP product line alongside M&amp;A - verify specific crypto issuance roles.</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>None - no restructuring practice</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>Mike Pascucci - Managing Director, CBS MBA '12</t>
         </is>
       </c>
-      <c r="I23" s="7" t="n"/>
+      <c r="K23" s="8" t="n"/>
     </row>
     <row r="24" ht="92" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1298,31 +1493,41 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
+          <t>Named: Digital Assets group</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
           <t>DIGITAL ASSETS GROUP within Cantor Fitzgerald &amp; Co. investment banking. Cantor Equity Partners (CEP, CEPT) are the affiliated SPAC sponsor vehicles. Bitcoin financing desk is separate again.</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>The deepest crypto ECM franchise in the market - if ECM genuinely interests you this is the highest-conviction name on the list. Be clear which arm you are targeting: advisory vs the SPAC sponsor vehicles vs bitcoin financing. Risk: DAT-lane concentration and the post-2025 derating of treasury companies.</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Semler Scientific ~$1.4B (buy-side FA to Strive, Sep 2025)</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Twenty One Capital (FA + placement, Apr 2025; NYSE: XXI Dec 2025 - the Tether/SoftBank vehicle); Securitize $1.25B pre-money (buy-side FA for CEPT, Oct 2025); bitcoin financing book</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="7" t="n"/>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="8" t="n"/>
     </row>
     <row r="25" ht="92" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -1337,35 +1542,45 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
+          <t>Named: Blockchain &amp; Digital Assets</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
           <t>BLOCKCHAIN &amp; DIGITAL ASSETS practice within Cohen &amp; Company Capital Markets (the IB arm). Distinct from Cohen &amp; Company Asset Management.</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Highest CBS alumni leverage of any firm on this list - an alum runs the practice you would be joining. Hiring is opportunistic (no structured program), so this is a relationship you build now and cash later. M&amp;A and ECM under one roof.</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Stronghold Digital $125M (sell-side, Aug 2024)</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>ProCap BTC ~$1B de-SPAC (exclusive FA + co-placement with Clear Street, Jun 2025; Nasdaq: BRR); Nakamoto ~$710M (lead FA + placement with 10X Capital, 2025)</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
         <is>
           <t>Christian J. Lopez - MD, HEAD of Blockchain &amp; Digital Assets, CBS MBA. Also Rahul Jasuja - MD, Energy &amp; Energy Transition IB, CBS MBA; Pawel Skonieczka - MD, CBS MBA '13</t>
         </is>
       </c>
-      <c r="I25" s="7" t="n"/>
+      <c r="K25" s="8" t="n"/>
     </row>
     <row r="26" ht="92" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -1380,31 +1595,41 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
+          <t>Named: FinTech &amp; Specialty Finance</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
           <t>FINANCIAL TECHNOLOGY &amp; SPECIALTY FINANCE group within KBW. Stifel's own investment bank is a separate platform (it ran the Riot mandate).</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>The premier FIG-only bank. Crypto work skews research and capital markets over M&amp;A - which is a FEATURE if ECM interests you. Bank-crypto convergence (charters, stablecoin issuers, exchange listings) could re-rate this seat quickly.</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>1 (Stifel's)</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Block Mining $92.5M (Stifel, excl. buy-side for Riot, Jul 2024)</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>FIG ECM is a core KBW franchise - the natural home for crypto-bank and stablecoin-issuer issuance. Verify specific roles.</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="7" t="n"/>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="8" t="n"/>
     </row>
     <row r="27" ht="92" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -1419,35 +1644,45 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
+          <t>ENTIRE FIRM</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
           <t>Broadhaven Capital Partners = the advisory arm (fintech and market structure). Broadhaven Ventures = the VC arm, same roof.</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>One relationship serves both your IB and VC lanes - the only firm on this list where that is true. Small team, lateral hiring, no junior program. Both founding partners are CBS.</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>1 (live mandate)</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>BitMEX sale mandate (process reported under way); ErisX to Cboe (historic market-structure credit)</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>Jerry von Dohlen - Founder &amp; Partner, CBS MBA '96 (+ Columbia Engineering BS); James Denton - Partner, CBS MBA '85</t>
         </is>
       </c>
-      <c r="I27" s="7" t="n"/>
+      <c r="K27" s="8" t="n"/>
     </row>
     <row r="28" ht="92" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -1462,31 +1697,41 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
+          <t>Crypto-native (whole firm)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
           <t>GALAXY DIGITAL PARTNERS = the investment banking / advisory arm. Distinct from Galaxy Ventures (VC), Galaxy Asset Management, Galaxy Global Markets (trading and lending), and Galaxy Data Centers (Helios).</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Largest crypto-native advisory platform; both mandates were exclusive sell-sides. Lateral hires and occasional postings - not an MBA summer program. One relationship opens IB and Ventures.</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Bitstamp $200M (excl. sell-side to Robinhood, Jun 2024); Aplo (excl. sell-side to Coincheck, Sep 2025, stock-for-stock)</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Galaxy Global Markets runs financing/structured products - adjacent to ECM but not underwriting.</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="7" t="n"/>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="8" t="n"/>
     </row>
     <row r="29" ht="92" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1501,31 +1746,41 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
+          <t>Crypto-native (whole firm)</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
           <t>Crypto-native M&amp;A advisory - senior-only team (~12 advisors), no departments, no junior program. Founder: Eric Risley.</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Their per-deal M&amp;A alerts name the advisors on every transaction in the market - engaging the research IS the relationship strategy. Treat as a 2029+ landing spot, not a recruiting target.</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>3+</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Coinme + Sequence ~$250M combined (excl. sell-side for Coinme to Polygon Labs, Jan 2026); Magic Labs wallet business (excl. sell-side to Payward, Jul 2026); Caleb &amp; Brown</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>No ECM practice.</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="7" t="n"/>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="8" t="n"/>
     </row>
     <row r="30" ht="92" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -1540,35 +1795,45 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
+          <t>Named: Blockchain &amp; Digital Infra</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
           <t>INVESTMENT BANKING - Blockchain &amp; Digital Infrastructure group. Sits alongside Clear Street's prime brokerage business.</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>A crypto-native-adjacent IB group run by a CBS alum, inside a prime broker - directly adjacent to your COR PRIME operating background. Growing platform.</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
         <is>
           <t>None disclosed as lead advisor</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>ProCap BTC ~$1B (co-placement agent with Cohen &amp; Co CM, Jun 2025)</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
         <is>
           <t>Collin Finnerty - MD, Blockchain &amp; Digital Infrastructure Investment Banking, CBS MBA '20</t>
         </is>
       </c>
-      <c r="I30" s="7" t="n"/>
+      <c r="K30" s="8" t="n"/>
     </row>
     <row r="31" ht="92" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -1583,35 +1848,45 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
+          <t>Within Technology / Business Svcs</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
           <t>Technology group (global co-head sits in NY) and Capital Advisory group. Mid-market focus.</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Nine CBS people including the CEO - the densest alumni cluster of any bank in the dataset - but a single crypto credit and a mid-market generalist mandate. An alumni-rich fallback, not a crypto thesis play.</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>GRIID Infrastructure $155M EV (sell-side FA + fairness opinion for CleanSpark, Jun 2024)</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Capital Advisory (private funds/GP advisory) - not crypto ECM.</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>Rob Brown - CEO, CBS MBA; Scott Twibell - MD Global Co-Head Technology; Steve Carre, Brian Goodwin, Mark Karasik, Mark Y. (MDs); Dave Reese (Director); Cole Ahnell (Associate, CBS '23); Mike Zhang (Analyst, CBS MS '24)</t>
         </is>
       </c>
-      <c r="I31" s="7" t="n"/>
+      <c r="K31" s="8" t="n"/>
     </row>
     <row r="32" ht="92" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -1626,31 +1901,41 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
+          <t>Within FIG</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
           <t>Investment Banking (small), FIG focus, research-led.</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>One real FA credit alongside Barclays. Lateral hiring only - watch postings.</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
         <is>
           <t>Long Ridge $1.5B (co-buy-side FA to MARA with Barclays, Apr 2026)</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Research-driven capital markets; verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="7" t="n"/>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="n"/>
+      <c r="K32" s="8" t="n"/>
     </row>
     <row r="33" ht="92" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -1665,31 +1950,41 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
+          <t>Bank-affiliated, no groups</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
           <t>Broker-dealer / investment banking arm of Cross River Bank.</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Early build-out of the franchise - small enough that one good conversation matters, and early joiners get outsized roles if the practice scales.</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>1 (co)</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>Reap up to $600M (co-sell-side with Goldman Sachs Asia for Payward, May 2026)</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="n"/>
-      <c r="I33" s="7" t="n"/>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="n"/>
+      <c r="K33" s="8" t="n"/>
     </row>
     <row r="34" ht="92" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -1704,31 +1999,41 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
+          <t>None - generalist</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
           <t>Independent generalist M&amp;A advisory.</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Single crypto credit; no dedicated digital-assets practice. Opportunistic only.</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>Block Mining $92.5M (excl. sell-side to Riot, Jul 2024)</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="7" t="n"/>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="n"/>
+      <c r="K34" s="8" t="n"/>
     </row>
     <row r="35" ht="92" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -1743,31 +2048,41 @@
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
+          <t>Crypto-native (whole firm)</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
           <t>Crypto-native M&amp;A advisory; Berlin HQ with Singapore and Dubai. No formal departments.</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Self-reports 15+ mandates in 2025 and $1B+ cumulative advised - these are the firm's own claims; verify mandate quality in conversation. Europe-weighted, smaller tickets. Fits your London/Europe base.</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>2 verified / 15+ self-reported</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
         <is>
           <t>Bulletin (sell-side); Bridgepoint / ht.digital (buy-side)</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="n"/>
-      <c r="I35" s="7" t="n"/>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="n"/>
+      <c r="K35" s="8" t="n"/>
     </row>
     <row r="36" ht="92" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -1782,31 +2097,41 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
+          <t>Named: Digital Assets group</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
           <t>DIGITAL ASSETS group; flow skews capital markets over M&amp;A.</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>A DCG-related mandate is referenced in the research but unnamed - treat as unverified. Lateral and just-in-time hiring.</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>0 verified</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>None verified</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>Digital assets capital markets is the stated franchise - verify specific issuance roles.</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="7" t="n"/>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="n"/>
+      <c r="K36" s="8" t="n"/>
     </row>
     <row r="37" ht="92" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -1821,31 +2146,41 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
+          <t>Named: Digital Assets</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
           <t>Digital Assets investment banking, research-led.</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>No disclosed M&amp;A credits 2024-26. Research and capital markets is the actual franchise. Lateral hiring.</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>Research-led digital assets capital markets - verify issuance roles.</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="7" t="n"/>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="n"/>
+      <c r="K37" s="8" t="n"/>
     </row>
     <row r="38" ht="92" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -1860,31 +2195,41 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
+          <t>Crypto-native (whole firm)</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
           <t>London digital-asset advisory boutique; no formal program.</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>No disclosed 2024-26 mandates surfaced in the research. Included for completeness and the London angle - verify the firm is active before spending time.</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>0 disclosed</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="7" t="n"/>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="n"/>
+      <c r="K38" s="8" t="n"/>
     </row>
     <row r="39" ht="92" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -1899,45 +2244,300 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
+          <t>Named: FinTech vertical</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
           <t>Technology M&amp;A boutique - FinTech vertical.</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>No crypto credit in the dataset, but a pure tech M&amp;A shop with a CBS MD. A fintech pitch, not a crypto one.</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>0 crypto / active fintech</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>None disclosed in crypto</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>Phillip Kim - Managing Director, CBS MBA '05; Joe Josephson - Partner (CBS '98)</t>
         </is>
       </c>
-      <c r="I39" s="7" t="n"/>
-    </row>
-    <row r="41" ht="100" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="K39" s="8" t="n"/>
+    </row>
+    <row r="40" ht="92" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Piper Sandler</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>FIG specialist</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>ENTIRE FIRM (FIG)</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Financial Services Group - FinTech coverage; absorbed Sandler O'Neill's FIG franchise.</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>The closest structural analogue to KBW and the biggest gap in your list. One of the deepest FIG franchises on the street. No crypto M&amp;A credit surfaced - this is a fintech pitch.</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>0 crypto / active fintech</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto; high-volume bank, specialty finance and payments M&amp;A</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>Major FIG ECM franchise - context only</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="n"/>
+      <c r="K40" s="8" t="n"/>
+    </row>
+    <row r="41" ht="92" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>William Blair</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Mid-market</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Named: FinTech / Payments</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Technology &amp; Services - FinTech and Payments coverage.</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Active upper-middle-market fintech and payments M&amp;A. No crypto credit surfaced.</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>0 crypto / active fintech</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto; recurring payments and fintech M&amp;A</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>Mid-market ECM - context only</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="n"/>
+      <c r="K41" s="8" t="n"/>
+    </row>
+    <row r="42" ht="92" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Raymond James</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>Mid-market</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Within Technology &amp; Services</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Investment Banking - Technology &amp; Services; FinTech coverage within it.</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Real fintech M&amp;A practice; no crypto credit surfaced.</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>0 crypto / active fintech</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>Mid-market ECM - context only</t>
+        </is>
+      </c>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="n"/>
+      <c r="K42" s="8" t="n"/>
+    </row>
+    <row r="43" ht="92" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>D.A. Davidson</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Mid-market</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Named: FinTech (ex-Marlin &amp; Associates team)</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Technology Investment Banking - FinTech group, built on the absorbed Marlin &amp; Associates team.</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Marlin was a dedicated fintech M&amp;A boutique before the acquisition - the team and franchise carried over. Mid-market.</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>0 crypto / active fintech</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto; fintech M&amp;A is the group's whole mandate</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>Limited</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J43" s="6" t="n"/>
+      <c r="K43" s="8" t="n"/>
+    </row>
+    <row r="44" ht="92" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Arma Partners</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>European tech specialist</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>ENTIRE FIRM (digital economy)</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Sector teams across the digital economy; FinTech is a core vertical. London-based.</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Europe's leading independent digital-economy adviser and a strong fit for your London base. No crypto credit surfaced - verify current crypto appetite.</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>0 crypto / active fintech</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto; heavy European fintech and software M&amp;A</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>No ECM - pure advisory</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="J44" s="6" t="n"/>
+      <c r="K44" s="8" t="n"/>
+    </row>
+    <row r="46" ht="100" customHeight="1">
+      <c r="A46" s="9" t="inlineStr">
         <is>
           <t>Deal mandates are advisor attributions verified from press releases, law-firm and bank announcements, SEC filings and Architect Partners M&amp;A alerts through Aug 21, 2026 — 'Not disclosed' on a transaction means no public attribution was found, not that no advisor was engaged, so several firms will have more credits than are listed. GROUP AND DEPARTMENT NAMES ARE FROM GENERAL KNOWLEDGE (Jan 2026 horizon) and banks rename and reorganize coverage groups constantly — confirm the exact group name on the firm's site or in your first conversation before using it. Items marked VERIFY are explicitly unconfirmed. ECM entries are thinner than M&amp;A across the board because underwriting syndicates are less consistently disclosed than advisory mandates; confirm bookrunner roles on the crypto IPO wave (Circle CRCL Jun 2025, Gemini GEMI Sep 2025, Bullish) directly from the prospectuses. Restructuring column is included so you can see which firms' crypto reputations rest entirely on estates work.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I39"/>
+  <autoFilter ref="A5:K44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 'OCR at CBS?' column to bank profiles
Splits the 39 firms into OCR (16: all seven BBs plus the nine elite
boutiques with structured summer associate programmes), non-OCR
(17: direct application, lateral or network-only), and verify (6).
Determines what competes for the Sept-Jan calendar.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WXzZsq4Qrn4tV9mBn34Mo
</commit_message>
<xml_diff>
--- a/IB_Target_Profiles.xlsx
+++ b/IB_Target_Profiles.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Profiles" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bank Profiles'!$A$5:$K$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bank Profiles'!$A$5:$L$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +115,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -483,12 +489,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="52" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -534,45 +540,50 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>OCR at CBS?</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
           <t>FinTech Coverage</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Group / Department to Target</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Department Notes &amp; Traps</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Crypto M&amp;A Credits</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Crypto &amp; Fintech M&amp;A Mandates</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>ECM / DAT / Capital Markets (context — not your target)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Restructuring (context — not your target)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>CBS Alumni Contact</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
@@ -589,43 +600,48 @@
           <t>Bulge bracket</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Global Banking &amp; Markets - Financial Institutions Group (FIG); fintech coverage sits in FIG/TMT. Separate Digital Assets team in GBM.</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Largest crypto M&amp;A count in the dataset, but crypto is a subset of a vast platform - you are recruiting into FIG, not into a crypto desk.</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>GTreasury $1B (excl. sell-side for Hg, Oct 2025); Core Scientific / CoreWeave $9B (buy-side, Jul 2025); Equiniti $4.2B (excl. buy-side for Bullish, May 2026); Reap up to $600M (co-sell, GS Asia, May 2026)</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Top-tier ECM franchise; crypto IPO wave (Circle CRCL Jun 2025, Bullish, Gemini GEMI Sep 2025) - VERIFY which bookrunner roles GS held. NEOS up to $2.25B was GS as principal buyer (GBM), not an advisory mandate.</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="8" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="8" t="n"/>
     </row>
     <row r="7" ht="92" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -638,47 +654,52 @@
           <t>Bulge bracket</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Named: FIG FinTech Coverage</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Investment Banking - FIG, FinTech coverage; Technology group adjacent.</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Most active BB in crypto by mandate count. Larger associate class than any EB. Leveraged finance sits alongside - the Long Ridge bridge came from the same relationship.</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Bitstamp $200M (excl. buy-side for Robinhood, Jun 2024); Long Ridge $1.5B (co-buy-side for MARA + bridge loan, Apr 2026); Kiavi $717M (excl. buy-side for Figure/Sixth Street, Jun 2026); NEOS up to $2.25B (excl. sell-side, Aug 2026)</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Long Ridge bridge financing (Apr 2026). Full ECM platform - confirm crypto/fintech issuance roles.</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
           <t>Taiwo O. - FIG FinTech Coverage, CBS MBA</t>
         </is>
       </c>
-      <c r="K7" s="8" t="n"/>
+      <c r="L7" s="8" t="n"/>
     </row>
     <row r="8" ht="92" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -691,43 +712,48 @@
           <t>Bulge bracket</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Dedicated FinTech coverage in IB</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Investment Banking - FIG / Financial Technology coverage.</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>TRAP: Kinexys (ex-Onyx) is JPM's blockchain PRODUCT unit - deposit tokens, tokenized repo. It is not investment banking and will not lead to an M&amp;A seat. Target FIG.</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Adecoagro ~$615.5M tender (excl. sell-side vs Tether, Mar 2025); WonderFi C$250M (buy-side for Robinhood, May 2025)</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Full ECM platform; reported role in the Circle (CRCL) IPO - VERIFY.</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="n"/>
-      <c r="K8" s="8" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="8" t="n"/>
     </row>
     <row r="9" ht="92" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -740,43 +766,48 @@
           <t>Bulge bracket</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Banking - FIG / Financial Technology; digital assets coverage within FIG.</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>TRAP: Citi Token Services is a product/treasury build, not IB. Citi's crypto credit is an ECM/DAT one, not M&amp;A.</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Securitize $1.25B pre-money de-SPAC (FA to Securitize + co-placement, Oct 2025; NYSE: SECZ Jul 2026)</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="n"/>
-      <c r="K9" s="8" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="8" t="n"/>
     </row>
     <row r="10" ht="92" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -789,47 +820,52 @@
           <t>Bulge bracket</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Named: Head of FinTech &amp; AI</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Investment Banking - Global Financial Institutions; FinTech coverage (Head of FinTech &amp; AI sits in London).</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto M&amp;A credit 2024-26. Included for fintech breadth and the E*TRADE crypto build. Verify before pitching crypto here.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>None disclosed in crypto. (Historic fintech/LatAm depth - Gol/Smiles was alongside MS, which is your own credential.)</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Full ECM platform - verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
           <t>Richard Pilipuitis - MD, Head of FinTech &amp; AI (CBS exec-ed, not a degree - soft tie)</t>
         </is>
       </c>
-      <c r="K10" s="8" t="n"/>
+      <c r="L10" s="8" t="n"/>
     </row>
     <row r="11" ht="92" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -842,47 +878,52 @@
           <t>Bulge bracket</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Investment Banking - Global FIG / FinTech; Technology group adjacent.</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto M&amp;A credit 2024-26. Fintech coverage is real; crypto is not a stated franchise.</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Full ECM platform - verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
           <t>Yusuf Ibrahim - IB Associate, fintech/tech, CBS MBA '25</t>
         </is>
       </c>
-      <c r="K11" s="8" t="n"/>
+      <c r="L11" s="8" t="n"/>
     </row>
     <row r="12" ht="92" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -895,43 +936,48 @@
           <t>Bulge bracket</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Corporate &amp; Investment Banking - FIG / Financial Technology.</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Single syndicate appearance; not a crypto franchise. Low priority unless a relationship appears.</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>1 (syndicate)</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Equiniti $4.2B (sell-side syndicate alongside Evercore/FT Partners leads, May 2026)</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="8" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="8" t="n"/>
     </row>
     <row r="13" ht="92" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -944,43 +990,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Within FIG (verify if branded)</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>STRATEGIC ADVISORY (M&amp;A). NOT RSSG.</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>CRITICAL: RSSG (Restructuring &amp; Special Situations Group) is a separate, MBA-heavy track and is where the Core Scientific Ch.11 sat - the tracks split early. Park Hill (fund placement) is a third arm. All the Payward M&amp;A work is Strategic Advisory. Say 'strategic advisory' in every conversation.</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>NinjaTrader $1.5B (buy-side for Kraken/Payward, Mar 2025); Core Scientific $9B (co-sell with Moelis, Jul 2025); Bitnomial up to $550M (excl. sell-side, Apr 2026); Reap up to $600M (buy-side for Payward, May 2026)</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Core Scientific Ch.11 debtors (RSSG) - context only</t>
         </is>
       </c>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="8" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="8" t="n"/>
     </row>
     <row r="14" ht="92" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -993,43 +1044,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR (consistent CBS hirer)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Advisory - FIG / Financial Technology coverage. Capital Markets Advisory (ECM) is a distinct group.</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Largest associate class among the EBs and a consistent CBS hirer. Crypto evidence is thin (one credit) - lead with the fintech franchise, not a crypto thesis.</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>Equiniti $4.2B (co-lead sell-side for Siris with FT Partners, May 2026)</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Capital Markets Advisory group; verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="8" t="n"/>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="8" t="n"/>
     </row>
     <row r="15" ht="92" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1042,43 +1098,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Generalist M&amp;A coverage. Recapitalization &amp; Restructuring (R&amp;R) is the separate arm.</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Its crypto reputation is 60% restructuring (Voyager, Genesis, BlockFi debtors). If you have ruled out Rx, only two of its five credits are relevant - and staffing can cross between M&amp;A and R&amp;R.</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Stronghold Digital $125M (buy-side for Bitfarms, Aug 2024); Core Scientific $9B (co-sell with PJT, Jul 2025)</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Genesis, Voyager, BlockFi debtors - context only</t>
         </is>
       </c>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="8" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="8" t="n"/>
     </row>
     <row r="16" ht="92" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1091,47 +1152,52 @@
           <t>Elite boutique / full platform</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR (largest class)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Named: FinTech &amp; Wealth</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Investment Banking - FINTECH &amp; WEALTH group (within FIG). Technology group adjacent. Full ECM platform in-house.</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Only firm combining three crypto M&amp;A sell-sides, real ECM, the largest associate class of the group, and a CBS alum leading the exact coverage group.</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>NinjaTrader $1.5B (sell-side, Mar 2025); Long Ridge $1.5B (co-sell with Lazard for FTAI, Apr 2026); Kiavi $717M (sell-side for Figure, Jun 2026)</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Full ECM/leveraged finance platform - the strongest ECM offering of any non-BB on this list. Verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>FTX creditors committee - context only</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>John Erwin - MD, FinTech &amp; Wealth Investment Banking, CBS MBA '06</t>
         </is>
       </c>
-      <c r="K16" s="8" t="n"/>
+      <c r="L16" s="8" t="n"/>
     </row>
     <row r="17" ht="92" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1144,43 +1210,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Financial Advisory - FIG; the Long Ridge mandate ran through Power &amp; Energy Infrastructure.</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Its single crypto credit was a POWER asset sale, not a crypto business - do not overstate it as a digital-assets franchise.</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>Long Ridge $1.5B (co-sell with Jefferies for FTAI, Apr 2026)</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="n"/>
-      <c r="K17" s="8" t="n"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="8" t="n"/>
     </row>
     <row r="18" ht="92" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1193,43 +1264,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR (smallest class)</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>None - generalist staffing</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Generalist advisory - no formal industry groups; industry-agnostic staffing.</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>ZERO crypto M&amp;A credits. Its only crypto work is the Celsius Ch.11 debtor role. Smallest class in the market.</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="G18" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Celsius Ch.11 debtors (~$20.1M fee allocation) - context only</t>
         </is>
       </c>
-      <c r="J18" s="6" t="n"/>
-      <c r="K18" s="8" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="8" t="n"/>
     </row>
     <row r="19" ht="92" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1242,43 +1318,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Single Advisory platform (M&amp;A and restructuring are not separately branded).</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>ZERO crypto M&amp;A credits. Both crypto engagements are restructuring - FTX debtors and Celsius creditors. Its crypto reputation is entirely estates.</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>FTX debtors (ran the LedgerX and FTX Europe sales); Celsius creditors - context only</t>
         </is>
       </c>
-      <c r="J19" s="6" t="n"/>
-      <c r="K19" s="8" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="8" t="n"/>
     </row>
     <row r="20" ht="92" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1291,43 +1372,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Named: FinTech (Corporate Finance)</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>CORPORATE FINANCE (M&amp;A) - has a real FinTech group. Financial Restructuring is the separate arm where the crypto work sat.</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>ZERO crypto M&amp;A credits; the Genesis role was creditor-side Rx. The Corporate Finance FinTech group is legitimate for fintech M&amp;A - but that is a fintech pitch, not a crypto one.</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>0 crypto / active fintech</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>None in crypto (Corporate Finance FinTech practice is active in payments/specialty finance broadly)</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Genesis creditors - context only</t>
         </is>
       </c>
-      <c r="J20" s="6" t="n"/>
-      <c r="K20" s="8" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="8" t="n"/>
     </row>
     <row r="21" ht="92" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1340,43 +1426,48 @@
           <t>Elite boutique</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Investment Banking - FIG / Technology coverage.</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto M&amp;A credits 2024-26 - the weakest evidence of any Tier 1 name. Only worth time if networking comes free.</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="n"/>
-      <c r="K21" s="8" t="n"/>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="8" t="n"/>
     </row>
     <row r="22" ht="92" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1389,43 +1480,48 @@
           <t>Merchant bank / boutique</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>NO — relationship-driven</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>None - TMT generalist</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Generalist merchant bank, TMT &amp; media focus; no dedicated crypto or fintech group.</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Founder-led (Aryeh Bourkoff), very small intake, relationship-driven. The Semler mandate shows real digital-asset appetite but arrived through generalist coverage.</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>Semler Scientific ~$1.4B all-stock (EXCLUSIVE sell-side vs Strive, Sep 2025 - the first DAT stock-for-stock merger); Equiniti $4.2B (sell-side syndicate, May 2026)</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="n"/>
-      <c r="K22" s="8" t="n"/>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="8" t="n"/>
     </row>
     <row r="23" ht="92" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -1438,47 +1534,52 @@
           <t>Fintech specialist</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>NO — direct via Greenhouse</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>ENTIRE FIRM</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>No traditional department structure - organized in vertical deal teams; the relevant vertical is Blockchain / Digital Assets. Founder-led (Steve McLaughlin).</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>The single purest fintech M&amp;A franchise on this list: 100% fintech, zero restructuring. Hires associates DIRECTLY via Greenhouse (no OCR), so it does not compete with your Sept-Jan calendar. Culture is famously demanding - diligence with former juniors before committing.</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>Hidden Road $1.25B (sell-side for Ripple, Apr 2025 - now Ripple Prime); Deribit $2.9B, $3.9-4.3B at close (sell-side for Coinbase, May 2025); WonderFi C$250M (sell-side, May 2025); Equiniti $4.2B (co-lead sell-side with Evercore, May 2026)</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Private capital raising is a core FTP product line alongside M&amp;A - verify specific crypto issuance roles.</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>None - no restructuring practice</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>Mike Pascucci - Managing Director, CBS MBA '12</t>
         </is>
       </c>
-      <c r="K23" s="8" t="n"/>
+      <c r="L23" s="8" t="n"/>
     </row>
     <row r="24" ht="92" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1491,43 +1592,48 @@
           <t>Full-service / DAT specialist</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>NO — posts roles, unstructured</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Named: Digital Assets group</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>DIGITAL ASSETS GROUP within Cantor Fitzgerald &amp; Co. investment banking. Cantor Equity Partners (CEP, CEPT) are the affiliated SPAC sponsor vehicles. Bitcoin financing desk is separate again.</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>The deepest crypto ECM franchise in the market - if ECM genuinely interests you this is the highest-conviction name on the list. Be clear which arm you are targeting: advisory vs the SPAC sponsor vehicles vs bitcoin financing. Risk: DAT-lane concentration and the post-2025 derating of treasury companies.</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>Semler Scientific ~$1.4B (buy-side FA to Strive, Sep 2025)</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Twenty One Capital (FA + placement, Apr 2025; NYSE: XXI Dec 2025 - the Tether/SoftBank vehicle); Securitize $1.25B pre-money (buy-side FA for CEPT, Oct 2025); bitcoin financing book</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="n"/>
-      <c r="K24" s="8" t="n"/>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="8" t="n"/>
     </row>
     <row r="25" ht="92" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -1540,47 +1646,52 @@
           <t>Boutique / DAT specialist</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>NO — opportunistic</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Named: Blockchain &amp; Digital Assets</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>BLOCKCHAIN &amp; DIGITAL ASSETS practice within Cohen &amp; Company Capital Markets (the IB arm). Distinct from Cohen &amp; Company Asset Management.</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Highest CBS alumni leverage of any firm on this list - an alum runs the practice you would be joining. Hiring is opportunistic (no structured program), so this is a relationship you build now and cash later. M&amp;A and ECM under one roof.</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>Stronghold Digital $125M (sell-side, Aug 2024)</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>ProCap BTC ~$1B de-SPAC (exclusive FA + co-placement with Clear Street, Jun 2025; Nasdaq: BRR); Nakamoto ~$710M (lead FA + placement with 10X Capital, 2025)</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
           <t>Christian J. Lopez - MD, HEAD of Blockchain &amp; Digital Assets, CBS MBA. Also Rahul Jasuja - MD, Energy &amp; Energy Transition IB, CBS MBA; Pawel Skonieczka - MD, CBS MBA '13</t>
         </is>
       </c>
-      <c r="K25" s="8" t="n"/>
+      <c r="L25" s="8" t="n"/>
     </row>
     <row r="26" ht="92" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -1593,43 +1704,48 @@
           <t>FIG specialist</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>NO — mostly lateral</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Named: FinTech &amp; Specialty Finance</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>FINANCIAL TECHNOLOGY &amp; SPECIALTY FINANCE group within KBW. Stifel's own investment bank is a separate platform (it ran the Riot mandate).</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>The premier FIG-only bank. Crypto work skews research and capital markets over M&amp;A - which is a FEATURE if ECM interests you. Bank-crypto convergence (charters, stablecoin issuers, exchange listings) could re-rate this seat quickly.</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>1 (Stifel's)</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Block Mining $92.5M (Stifel, excl. buy-side for Riot, Jul 2024)</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>FIG ECM is a core KBW franchise - the natural home for crypto-bank and stablecoin-issuer issuance. Verify specific roles.</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="n"/>
-      <c r="K26" s="8" t="n"/>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="8" t="n"/>
     </row>
     <row r="27" ht="92" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -1642,47 +1758,52 @@
           <t>Fintech / market-structure specialist</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>NO — small team, lateral</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>ENTIRE FIRM</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Broadhaven Capital Partners = the advisory arm (fintech and market structure). Broadhaven Ventures = the VC arm, same roof.</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>One relationship serves both your IB and VC lanes - the only firm on this list where that is true. Small team, lateral hiring, no junior program. Both founding partners are CBS.</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>1 (live mandate)</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>BitMEX sale mandate (process reported under way); ErisX to Cboe (historic market-structure credit)</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
           <t>Jerry von Dohlen - Founder &amp; Partner, CBS MBA '96 (+ Columbia Engineering BS); James Denton - Partner, CBS MBA '85</t>
         </is>
       </c>
-      <c r="K27" s="8" t="n"/>
+      <c r="L27" s="8" t="n"/>
     </row>
     <row r="28" ht="92" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -1695,43 +1816,48 @@
           <t>Crypto-native advisory</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>NO — lateral, occasional postings</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Crypto-native (whole firm)</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>GALAXY DIGITAL PARTNERS = the investment banking / advisory arm. Distinct from Galaxy Ventures (VC), Galaxy Asset Management, Galaxy Global Markets (trading and lending), and Galaxy Data Centers (Helios).</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Largest crypto-native advisory platform; both mandates were exclusive sell-sides. Lateral hires and occasional postings - not an MBA summer program. One relationship opens IB and Ventures.</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Bitstamp $200M (excl. sell-side to Robinhood, Jun 2024); Aplo (excl. sell-side to Coincheck, Sep 2025, stock-for-stock)</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>Galaxy Global Markets runs financing/structured products - adjacent to ECM but not underwriting.</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="n"/>
-      <c r="K28" s="8" t="n"/>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="8" t="n"/>
     </row>
     <row r="29" ht="92" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1744,43 +1870,48 @@
           <t>Crypto-native advisory</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>NO — no junior programme</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Crypto-native (whole firm)</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Crypto-native M&amp;A advisory - senior-only team (~12 advisors), no departments, no junior program. Founder: Eric Risley.</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Their per-deal M&amp;A alerts name the advisors on every transaction in the market - engaging the research IS the relationship strategy. Treat as a 2029+ landing spot, not a recruiting target.</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>3+</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>Coinme + Sequence ~$250M combined (excl. sell-side for Coinme to Polygon Labs, Jan 2026); Magic Labs wallet business (excl. sell-side to Payward, Jul 2026); Caleb &amp; Brown</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>No ECM practice.</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="n"/>
-      <c r="K29" s="8" t="n"/>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="n"/>
+      <c r="L29" s="8" t="n"/>
     </row>
     <row r="30" ht="92" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -1793,47 +1924,52 @@
           <t>Prime broker with IB arm</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>VERIFY — growing platform</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>Named: Blockchain &amp; Digital Infra</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>INVESTMENT BANKING - Blockchain &amp; Digital Infrastructure group. Sits alongside Clear Street's prime brokerage business.</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>A crypto-native-adjacent IB group run by a CBS alum, inside a prime broker - directly adjacent to your COR PRIME operating background. Growing platform.</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>None disclosed as lead advisor</t>
         </is>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="I30" s="6" t="inlineStr">
         <is>
           <t>ProCap BTC ~$1B (co-placement agent with Cohen &amp; Co CM, Jun 2025)</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
           <t>Collin Finnerty - MD, Blockchain &amp; Digital Infrastructure Investment Banking, CBS MBA '20</t>
         </is>
       </c>
-      <c r="K30" s="8" t="n"/>
+      <c r="L30" s="8" t="n"/>
     </row>
     <row r="31" ht="92" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -1846,47 +1982,52 @@
           <t>Mid-market</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>VERIFY — has hired CBS MBA associates</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Within Technology / Business Svcs</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Technology group (global co-head sits in NY) and Capital Advisory group. Mid-market focus.</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Nine CBS people including the CEO - the densest alumni cluster of any bank in the dataset - but a single crypto credit and a mid-market generalist mandate. An alumni-rich fallback, not a crypto thesis play.</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>GRIID Infrastructure $155M EV (sell-side FA + fairness opinion for CleanSpark, Jun 2024)</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Capital Advisory (private funds/GP advisory) - not crypto ECM.</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
           <t>Rob Brown - CEO, CBS MBA; Scott Twibell - MD Global Co-Head Technology; Steve Carre, Brian Goodwin, Mark Karasik, Mark Y. (MDs); Dave Reese (Director); Cole Ahnell (Associate, CBS '23); Mike Zhang (Analyst, CBS MS '24)</t>
         </is>
       </c>
-      <c r="K31" s="8" t="n"/>
+      <c r="L31" s="8" t="n"/>
     </row>
     <row r="32" ht="92" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -1899,43 +2040,48 @@
           <t>Research-led boutique</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>NO — lateral</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Within FIG</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Investment Banking (small), FIG focus, research-led.</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>One real FA credit alongside Barclays. Lateral hiring only - watch postings.</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="G32" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>Long Ridge $1.5B (co-buy-side FA to MARA with Barclays, Apr 2026)</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>Research-driven capital markets; verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="n"/>
-      <c r="K32" s="8" t="n"/>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="n"/>
+      <c r="L32" s="8" t="n"/>
     </row>
     <row r="33" ht="92" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -1948,43 +2094,48 @@
           <t>Bank-affiliated broker-dealer</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>NO — early build-out</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Bank-affiliated, no groups</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Broker-dealer / investment banking arm of Cross River Bank.</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Early build-out of the franchise - small enough that one good conversation matters, and early joiners get outsized roles if the practice scales.</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>1 (co)</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>Reap up to $600M (co-sell-side with Goldman Sachs Asia for Payward, May 2026)</t>
         </is>
       </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="8" t="n"/>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="n"/>
+      <c r="L33" s="8" t="n"/>
     </row>
     <row r="34" ht="92" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -1997,43 +2148,48 @@
           <t>Independent advisory</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>NO — small/opportunistic</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>None - generalist</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>Independent generalist M&amp;A advisory.</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Single crypto credit; no dedicated digital-assets practice. Opportunistic only.</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>Block Mining $92.5M (excl. sell-side to Riot, Jul 2024)</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
+      <c r="I34" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="n"/>
-      <c r="K34" s="8" t="n"/>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="n"/>
+      <c r="L34" s="8" t="n"/>
     </row>
     <row r="35" ht="92" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -2046,43 +2202,48 @@
           <t>Crypto-native advisory (Europe)</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>NO — no formal programme</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Crypto-native (whole firm)</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Crypto-native M&amp;A advisory; Berlin HQ with Singapore and Dubai. No formal departments.</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Self-reports 15+ mandates in 2025 and $1B+ cumulative advised - these are the firm's own claims; verify mandate quality in conversation. Europe-weighted, smaller tickets. Fits your London/Europe base.</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>2 verified / 15+ self-reported</t>
         </is>
       </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>Bulletin (sell-side); Bridgepoint / ht.digital (buy-side)</t>
         </is>
       </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J35" s="6" t="n"/>
-      <c r="K35" s="8" t="n"/>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K35" s="6" t="n"/>
+      <c r="L35" s="8" t="n"/>
     </row>
     <row r="36" ht="92" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -2095,43 +2256,48 @@
           <t>Mid-market / capital markets</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>NO — lateral / just-in-time</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>Named: Digital Assets group</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>DIGITAL ASSETS group; flow skews capital markets over M&amp;A.</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>A DCG-related mandate is referenced in the research but unnamed - treat as unverified. Lateral and just-in-time hiring.</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>0 verified</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>None verified</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="I36" s="6" t="inlineStr">
         <is>
           <t>Digital assets capital markets is the stated franchise - verify specific issuance roles.</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J36" s="6" t="n"/>
-      <c r="K36" s="8" t="n"/>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="8" t="n"/>
     </row>
     <row r="37" ht="92" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -2144,43 +2310,48 @@
           <t>Research-led broker-dealer</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>NO — lateral</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Named: Digital Assets</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Digital Assets investment banking, research-led.</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>No disclosed M&amp;A credits 2024-26. Research and capital markets is the actual franchise. Lateral hiring.</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="I37" s="6" t="inlineStr">
         <is>
           <t>Research-led digital assets capital markets - verify issuance roles.</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J37" s="6" t="n"/>
-      <c r="K37" s="8" t="n"/>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="n"/>
+      <c r="L37" s="8" t="n"/>
     </row>
     <row r="38" ht="92" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -2193,43 +2364,48 @@
           <t>Crypto-native advisory (London)</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>NO — no formal programme</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>Crypto-native (whole firm)</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>London digital-asset advisory boutique; no formal program.</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>No disclosed 2024-26 mandates surfaced in the research. Included for completeness and the London angle - verify the firm is active before spending time.</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>0 disclosed</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
+      <c r="I38" s="6" t="inlineStr">
         <is>
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="n"/>
-      <c r="K38" s="8" t="n"/>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K38" s="6" t="n"/>
+      <c r="L38" s="8" t="n"/>
     </row>
     <row r="39" ht="92" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -2242,47 +2418,52 @@
           <t>Technology specialist</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>VERIFY — small, likely direct</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Named: FinTech vertical</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Technology M&amp;A boutique - FinTech vertical.</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>No crypto credit in the dataset, but a pure tech M&amp;A shop with a CBS MD. A fintech pitch, not a crypto one.</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="G39" s="7" t="inlineStr">
         <is>
           <t>0 crypto / active fintech</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>None disclosed in crypto</t>
         </is>
       </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="I39" s="6" t="inlineStr">
         <is>
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K39" s="6" t="inlineStr">
+        <is>
           <t>Phillip Kim - Managing Director, CBS MBA '05; Joe Josephson - Partner (CBS '98)</t>
         </is>
       </c>
-      <c r="K39" s="8" t="n"/>
+      <c r="L39" s="8" t="n"/>
     </row>
     <row r="40" ht="92" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -2295,43 +2476,48 @@
           <t>FIG specialist</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>VERIFY — runs MBA recruiting; confirm CBS</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>ENTIRE FIRM (FIG)</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>Financial Services Group - FinTech coverage; absorbed Sandler O'Neill's FIG franchise.</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>The closest structural analogue to KBW and the biggest gap in your list. One of the deepest FIG franchises on the street. No crypto M&amp;A credit surfaced - this is a fintech pitch.</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>0 crypto / active fintech</t>
         </is>
       </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>None surfaced in crypto; high-volume bank, specialty finance and payments M&amp;A</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>Major FIG ECM franchise - context only</t>
         </is>
       </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J40" s="6" t="n"/>
-      <c r="K40" s="8" t="n"/>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K40" s="6" t="n"/>
+      <c r="L40" s="8" t="n"/>
     </row>
     <row r="41" ht="92" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -2344,43 +2530,48 @@
           <t>Mid-market</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>VERIFY — has MBA summer associate programme; confirm CBS</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Named: FinTech / Payments</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Technology &amp; Services - FinTech and Payments coverage.</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Active upper-middle-market fintech and payments M&amp;A. No crypto credit surfaced.</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="G41" s="7" t="inlineStr">
         <is>
           <t>0 crypto / active fintech</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>None surfaced in crypto; recurring payments and fintech M&amp;A</t>
         </is>
       </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="I41" s="6" t="inlineStr">
         <is>
           <t>Mid-market ECM - context only</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="n"/>
-      <c r="K41" s="8" t="n"/>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K41" s="6" t="n"/>
+      <c r="L41" s="8" t="n"/>
     </row>
     <row r="42" ht="92" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2393,43 +2584,48 @@
           <t>Mid-market</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>VERIFY — has MBA associate programme; confirm CBS</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Within Technology &amp; Services</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>Investment Banking - Technology &amp; Services; FinTech coverage within it.</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>Real fintech M&amp;A practice; no crypto credit surfaced.</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>0 crypto / active fintech</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>None surfaced in crypto</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="I42" s="6" t="inlineStr">
         <is>
           <t>Mid-market ECM - context only</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J42" s="6" t="n"/>
-      <c r="K42" s="8" t="n"/>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K42" s="6" t="n"/>
+      <c r="L42" s="8" t="n"/>
     </row>
     <row r="43" ht="92" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -2442,43 +2638,48 @@
           <t>Mid-market</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>NO — small MBA intake</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Named: FinTech (ex-Marlin &amp; Associates team)</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>Technology Investment Banking - FinTech group, built on the absorbed Marlin &amp; Associates team.</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Marlin was a dedicated fintech M&amp;A boutique before the acquisition - the team and franchise carried over. Mid-market.</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
+      <c r="G43" s="7" t="inlineStr">
         <is>
           <t>0 crypto / active fintech</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>None surfaced in crypto; fintech M&amp;A is the group's whole mandate</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="I43" s="6" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J43" s="6" t="n"/>
-      <c r="K43" s="8" t="n"/>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K43" s="6" t="n"/>
+      <c r="L43" s="8" t="n"/>
     </row>
     <row r="44" ht="92" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -2491,44 +2692,50 @@
           <t>European tech specialist</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>NO — European, no US OCR</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>ENTIRE FIRM (digital economy)</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>Sector teams across the digital economy; FinTech is a core vertical. London-based.</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Europe's leading independent digital-economy adviser and a strong fit for your London base. No crypto credit surfaced - verify current crypto appetite.</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
+      <c r="G44" s="7" t="inlineStr">
         <is>
           <t>0 crypto / active fintech</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>None surfaced in crypto; heavy European fintech and software M&amp;A</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="I44" s="6" t="inlineStr">
         <is>
           <t>No ECM - pure advisory</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="J44" s="6" t="n"/>
-      <c r="K44" s="8" t="n"/>
-    </row>
+      <c r="J44" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto</t>
+        </is>
+      </c>
+      <c r="K44" s="6" t="n"/>
+      <c r="L44" s="8" t="n"/>
+    </row>
+    <row r="45"/>
     <row r="46" ht="100" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
@@ -2537,7 +2744,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:K44"/>
+  <autoFilter ref="A5:L44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Ranked Targets tab; strip restructuring from profiles
- New Ranked Targets tab: 25 firms ranked on deal flow x access x
  alumni, with FT Partners / Jefferies / Galaxy at the top per George's
  call, an OCR at CBS column, and the exact group to apply for at each
- Removed the restructuring column and scrubbed Rx language from Bank
  Profiles; kept only the PJT Strategic-Advisory-not-RSSG guardrail

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WXzZsq4Qrn4tV9mBn34Mo
</commit_message>
<xml_diff>
--- a/IB_Target_Profiles.xlsx
+++ b/IB_Target_Profiles.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Profiles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ranked Targets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bank Profiles" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bank Profiles'!$A$5:$L$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ranked Targets'!$A$5:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bank Profiles'!$A$5:$K$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +61,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF7E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -94,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,6 +129,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -485,11 +504,1008 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FFC00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ranked Targets — Crypto &amp; FinTech M&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>M&amp;A only. Ranked on deal flow x access x alumni door, with your three priorities at the top. Full profiles on the Bank Profiles tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="13.5" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Fill in 'Your Notes' yourself. OCR firms compete for the Sept–Jan calendar; non-OCR firms run rolling and are additive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1"/>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Bank / Boutique</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>OCR at CBS?</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>GROUP TO APPLY FOR</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Why this rank</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Crypto &amp; FinTech M&amp;A Deal Flow</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>CBS Alumni Contact</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Your Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="96" customHeight="1">
+      <c r="A6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>FT Partners (Financial Technology Partners)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>NO — direct application via Greenhouse</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Investment Banking associate programme; ask for the BLOCKCHAIN / DIGITAL ASSETS vertical. No departments — the firm organises in deal teams.</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>YOUR PICK. The purest fit on the list: four crypto M&amp;A sell-sides, 100% fintech, no other business lines diluting the work. Applies outside OCR so it costs you nothing in Sept–Jan. Diligence the culture with former juniors before committing.</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Hidden Road $1.25B (sell, Ripple, Apr 2025); Deribit $2.9B (sell, Coinbase, May 2025); WonderFi C$250M (sell, May 2025); Equiniti $4.2B (co-lead sell, May 2026)</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Mike Pascucci — Managing Director, CBS MBA '12</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="96" customHeight="1">
+      <c r="A7" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Jefferies</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>YES — OCR (largest associate class)</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Investment Banking — FINTECH &amp; WEALTH group (sits within FIG).</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>YOUR PICK, and the one that carries the summer-2027 seat: the other two priorities cannot give you a structured internship. Three crypto sell-sides, a named fintech group, the biggest class of the group, and a CBS alum running that exact team.</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>NinjaTrader $1.5B (sell, Mar 2025); Long Ridge $1.5B (co-sell, Apr 2026); Kiavi $717M (sell, Figure, Jun 2026)</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>John Erwin — MD, FinTech &amp; Wealth Investment Banking, CBS MBA '06</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="96" customHeight="1">
+      <c r="A8" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Galaxy Digital Partners</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>NO — lateral hires, occasional postings</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>GALAXY DIGITAL PARTNERS — the investment banking / advisory arm. NOT Galaxy Ventures, NOT Asset Management, NOT Global Markets, NOT Data Centers.</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>YOUR PICK. Largest crypto-native advisory platform and both mandates were exclusive sell-sides. One relationship opens IB and Ventures. Timing: post-Optimus close, spring 2027.</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Bitstamp $200M (excl. sell to Robinhood, Jun 2024); Aplo (excl. sell to Coincheck, Sep 2025)</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="96" customHeight="1">
+      <c r="A9" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Barclays</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Investment Banking — FIG, FINTECH COVERAGE.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Most active bulge bracket in crypto by M&amp;A count, a named fintech group, a CBS alum sitting in it, and a bigger class than any boutique. Gives you fintech breadth if crypto cools in 2027.</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Bitstamp $200M (buy, Jun 2024); Long Ridge $1.5B (co-buy + bridge, Apr 2026); Kiavi $717M (excl. buy, Jun 2026); NEOS $2.25B (excl. sell, Aug 2026)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Taiwo O. — FIG FinTech Coverage, CBS MBA</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="96" customHeight="1">
+      <c r="A10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>PJT Partners</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>STRATEGIC ADVISORY (the M&amp;A arm). PJT also has RSSG, Park Hill and Camberview — separate tracks. Say 'strategic advisory' every time.</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Highest crypto M&amp;A credit count of any elite boutique, all through the Payward relationship. No alumni door, so you win it on thesis and IBC advocates.</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>NinjaTrader $1.5B (buy, Kraken, Mar 2025); Core Scientific $9B (co-sell, Jul 2025); Bitnomial $550M (excl. sell, Apr 2026); Reap $600M (buy, May 2026)</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="n"/>
+    </row>
+    <row r="11" ht="96" customHeight="1">
+      <c r="A11" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Goldman Sachs</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Global Banking &amp; Markets — FIG; ask for fintech / digital-assets coverage within FIG.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Most crypto M&amp;A credits in the dataset and the biggest tickets. Hardest door on the list — worth one advocate, not a campaign.</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>GTreasury $1B (excl. sell for Hg, Oct 2025); Core Scientific $9B (buy, CoreWeave, Jul 2025); Equiniti $4.2B (excl. buy, Bullish, May 2026); Reap $600M (co-sell Asia, May 2026)</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="96" customHeight="1">
+      <c r="A12" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Evercore</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR (consistent CBS hirer)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Advisory — FIG; ask to be pointed at the fintech bankers.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Your odds hedge: largest EB associate class and a reliable CBS hirer. Only one crypto credit, so lead with the fintech franchise and Gol/Smiles, not a crypto thesis.</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Equiniti $4.2B (co-lead sell for Siris with FT Partners, May 2026)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="96" customHeight="1">
+      <c r="A13" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Broadhaven Capital Partners</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>NO — small team, lateral</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>BROADHAVEN CAPITAL PARTNERS (the advisory arm). Broadhaven Ventures is the separate VC arm under the same roof.</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Pure fintech and market-structure M&amp;A, and the only firm where one relationship serves your IB and VC lanes at once. Both founding partners are CBS.</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>BitMEX sale mandate (live process); ErisX to Cboe (historic market-structure credit)</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Jerry von Dohlen — Founder &amp; Partner, CBS MBA '96; James Denton — Partner, CBS MBA '85</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="n"/>
+    </row>
+    <row r="14" ht="96" customHeight="1">
+      <c r="A14" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Cohen &amp; Company Capital Markets</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>NO — opportunistic hiring</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>COHEN &amp; COMPANY CAPITAL MARKETS (CCM) — Blockchain &amp; Digital Assets practice. NOT Cohen &amp; Company Asset Management.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>The best alumni door in your IB lane — an alum heads the practice. But the work is de-SPAC structuring and PIPE placement with one true sell-side; ask Lopez directly whether the group runs strategic M&amp;A beyond the DAT lane.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Stronghold Digital $125M (sell, Aug 2024)</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Christian J. Lopez — MD, HEAD of Blockchain &amp; Digital Assets, CBS MBA; Rahul Jasuja — MD, CBS MBA</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="96" customHeight="1">
+      <c r="A15" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Architect Partners</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>NO — no junior programme</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>No departments — senior-only partnership (~12 advisers). Approach the partners directly.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Three exclusive crypto sell-sides and the best mid-market crypto franchise, but no seat for you now. Engage the M&amp;A alerts — that research IS the relationship. A 2029+ landing spot.</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Coinme + Sequence ~$250M (excl. sell, Jan 2026); Magic Labs wallet business (excl. sell, Jul 2026); Caleb &amp; Brown</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="96" customHeight="1">
+      <c r="A16" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Houlihan Lokey</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>CORPORATE FINANCE — FinTech group. (Corporate Finance is the M&amp;A division.)</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>#1 globally in M&amp;A by deal count and mid-market focused, which matches where most crypto deals actually clear. Zero crypto credits — a fintech pitch only.</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto; high-volume mid-market fintech M&amp;A</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="n"/>
+    </row>
+    <row r="17" ht="96" customHeight="1">
+      <c r="A17" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>LionTree</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>NO — relationship-driven</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Generalist merchant bank, TMT and media focus. No fintech or crypto group — approach the firm, not a desk.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Ran the exclusive Semler sell-side, the first DAT stock-for-stock merger. Real digital-asset appetite but a very small intake.</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Semler Scientific ~$1.4B (EXCL. sell vs Strive, Sep 2025); Equiniti $4.2B (sell syndicate, May 2026)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="n"/>
+    </row>
+    <row r="18" ht="96" customHeight="1">
+      <c r="A18" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Moelis</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Investment Banking — FIG (generalist M&amp;A coverage).</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Two crypto M&amp;A credits and full OCR access. Solid, not differentiated — no named fintech group and no alumni door.</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Stronghold Digital $125M (buy, Bitfarms, Aug 2024); Core Scientific $9B (co-sell with PJT, Jul 2025)</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="96" customHeight="1">
+      <c r="A19" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>JPMorgan</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Investment Banking — FIG, FINANCIAL TECHNOLOGY coverage. (Kinexys is a product unit, not IB — do not target it.)</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Dedicated fintech coverage and a huge platform. Note the Adecoagro mandate came from LatAm/agri coverage, not fintech — so the crypto flow into the fintech team is thinner than the credit count suggests.</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Adecoagro ~$615.5M (excl. sell vs Tether, Mar 2025); WonderFi C$250M (buy, Robinhood, May 2025)</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="n"/>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Clear Street</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>VERIFY — growing platform</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Investment Banking — BLOCKCHAIN &amp; DIGITAL INFRASTRUCTURE group.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>A crypto-native IB group run by a CBS alum inside a prime broker — directly adjacent to your COR PRIME operating background. No lead M&amp;A credit yet.</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>None as lead adviser; co-placement on ProCap ~$1B (Jun 2025)</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Collin Finnerty — MD, Blockchain &amp; Digital Infrastructure IB, CBS MBA '20</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="n"/>
+    </row>
+    <row r="21" ht="96" customHeight="1">
+      <c r="A21" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Piper Sandler</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>VERIFY — runs MBA recruiting; confirm CBS</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Financial Services Group — FinTech coverage (built on the absorbed Sandler O'Neill FIG franchise).</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>One of the deepest FIG franchises on the street and the biggest gap in your original list. No crypto credit — a fintech pitch.</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto; high-volume bank, specialty finance and payments M&amp;A</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="96" customHeight="1">
+      <c r="A22" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Lazard</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Financial Advisory — FIG.</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>One credit, and it came through Power &amp; Energy Infrastructure (FTAI was a power asset), not a digital-assets franchise. Portfolio filler.</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Long Ridge $1.5B (co-sell for FTAI, Apr 2026)</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="96" customHeight="1">
+      <c r="A23" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Union Square Advisors</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>VERIFY — small, likely direct</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Technology M&amp;A — FINTECH vertical.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Pure tech M&amp;A boutique with a CBS MD. No crypto credit — fintech framing only.</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>None disclosed in crypto</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Phillip Kim — Managing Director, CBS MBA '05</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="n"/>
+    </row>
+    <row r="24" ht="96" customHeight="1">
+      <c r="A24" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>William Blair</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>VERIFY — has MBA summer associate programme; confirm CBS</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Technology &amp; Services — FINTECH / PAYMENTS coverage.</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Active upper-middle-market fintech and payments M&amp;A. No crypto credit.</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto; recurring payments and fintech M&amp;A</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="n"/>
+    </row>
+    <row r="25" ht="96" customHeight="1">
+      <c r="A25" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Lincoln International</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>VERIFY — has hired CBS MBA associates</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Technology group (fintech sits within Technology / Business Services).</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Nine CBS people including the CEO — the densest alumni cluster of any bank here — but one crypto credit and a mid-market generalist mandate.</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>GRIID Infrastructure $155M (sell FA + fairness opinion, CleanSpark, Jun 2024)</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Rob Brown — CEO, CBS MBA; Cole Ahnell — Associate, CBS '23; plus 7 more</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="n"/>
+    </row>
+    <row r="26" ht="96" customHeight="1">
+      <c r="A26" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Arma Partners</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>NO — European, no US OCR</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>FinTech sector team (London).</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Europe's leading independent digital-economy adviser and a natural fit for your London network. No crypto credit surfaced.</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>None surfaced in crypto; heavy European fintech and software M&amp;A</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="n"/>
+    </row>
+    <row r="27" ht="96" customHeight="1">
+      <c r="A27" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Cantor Fitzgerald</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>NO — posts roles, unstructured</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>DIGITAL ASSETS group within Cantor Fitzgerald &amp; Co. investment banking.</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Named digital-assets group, but the franchise is capital markets and DAT vehicles — only one M&amp;A credit. Low priority on an M&amp;A-only mandate.</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Semler Scientific ~$1.4B (buy-side FA to Strive, Sep 2025)</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="n"/>
+    </row>
+    <row r="28" ht="96" customHeight="1">
+      <c r="A28" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Morgan Stanley</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Investment Banking — Global Financial Institutions, FINTECH coverage.</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Named fintech leadership and a top-tier platform, but zero crypto M&amp;A credits. OCR breadth option.</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>None disclosed in crypto</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="n"/>
+    </row>
+    <row r="29" ht="96" customHeight="1">
+      <c r="A29" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Citigroup</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Banking — FIG, Financial Technology. (Citi Token Services is a product build, not IB.)</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Zero crypto M&amp;A — its only crypto credit is capital markets. OCR breadth option only.</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>None in crypto M&amp;A</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="n"/>
+    </row>
+    <row r="30" ht="96" customHeight="1">
+      <c r="A30" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Bank of America</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>YES — OCR</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Investment Banking — Global FIG, FinTech coverage.</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>No crypto credit; real fintech coverage. OCR breadth option, and there is a CBS associate inside to talk to.</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>None disclosed in crypto</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>Yusuf Ibrahim — IB Associate, fintech/tech, CBS MBA '25</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="n"/>
+    </row>
+    <row r="32" ht="74" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Rows 1–3 are your stated priorities (gold). Ranking below that weighs crypto/fintech M&amp;A deal flow, structural access, and whether a CBS alum sits inside. OCR status reflects general MBA-recruiting patterns and your Aug 2026 tracker research — CBS's actual 2026-27 OCR employer roster lives on the CMC portal and firms move on and off school lists every year, so reconcile this column in week one before committing your autumn. Group names are general knowledge (Jan 2026 horizon); banks rename coverage groups constantly, so confirm the exact name before using it in an email. Deal attributions are from press releases, law-firm and bank announcements, SEC filings and Architect Partners alerts through Aug 21, 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:H30"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FF1F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -575,15 +1591,10 @@
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Restructuring (context — not your target)</t>
+          <t>CBS Alumni Contact</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>CBS Alumni Contact</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
@@ -635,13 +1646,8 @@
           <t>Top-tier ECM franchise; crypto IPO wave (Circle CRCL Jun 2025, Bullish, Gemini GEMI Sep 2025) - VERIFY which bookrunner roles GS held. NEOS up to $2.25B was GS as principal buyer (GBM), not an advisory mandate.</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="8" t="n"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="8" t="n"/>
     </row>
     <row r="7" ht="92" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -691,15 +1697,10 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
           <t>Taiwo O. - FIG FinTech Coverage, CBS MBA</t>
         </is>
       </c>
-      <c r="L7" s="8" t="n"/>
+      <c r="K7" s="8" t="n"/>
     </row>
     <row r="8" ht="92" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -747,13 +1748,8 @@
           <t>Full ECM platform; reported role in the Circle (CRCL) IPO - VERIFY.</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="8" t="n"/>
+      <c r="J8" s="6" t="n"/>
+      <c r="K8" s="8" t="n"/>
     </row>
     <row r="9" ht="92" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -801,13 +1797,8 @@
           <t>Securitize $1.25B pre-money de-SPAC (FA to Securitize + co-placement, Oct 2025; NYSE: SECZ Jul 2026)</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="8" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="8" t="n"/>
     </row>
     <row r="10" ht="92" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -857,15 +1848,10 @@
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
           <t>Richard Pilipuitis - MD, Head of FinTech &amp; AI (CBS exec-ed, not a degree - soft tie)</t>
         </is>
       </c>
-      <c r="L10" s="8" t="n"/>
+      <c r="K10" s="8" t="n"/>
     </row>
     <row r="11" ht="92" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -915,15 +1901,10 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
           <t>Yusuf Ibrahim - IB Associate, fintech/tech, CBS MBA '25</t>
         </is>
       </c>
-      <c r="L11" s="8" t="n"/>
+      <c r="K11" s="8" t="n"/>
     </row>
     <row r="12" ht="92" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -971,13 +1952,8 @@
           <t>Verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="8" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="8" t="n"/>
     </row>
     <row r="13" ht="92" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -1002,7 +1978,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>STRATEGIC ADVISORY (M&amp;A). NOT RSSG.</t>
+          <t>CRITICAL: PJT has four arms — Strategic Advisory (M&amp;A, your target), RSSG, Park Hill (fund placement) and Camberview (shareholder advisory). All the Payward M&amp;A work is Strategic Advisory. Say 'strategic advisory' in every conversation so you are not routed elsewhere.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1025,13 +2001,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Core Scientific Ch.11 debtors (RSSG) - context only</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="8" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="8" t="n"/>
     </row>
     <row r="14" ht="92" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1079,13 +2050,8 @@
           <t>Capital Markets Advisory group; verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="8" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="8" t="n"/>
     </row>
     <row r="15" ht="92" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -1110,7 +2076,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Generalist M&amp;A coverage. Recapitalization &amp; Restructuring (R&amp;R) is the separate arm.</t>
+          <t>Generalist FIG / M&amp;A coverage with two crypto M&amp;A credits. Associate staffing is broad across the platform.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1133,13 +2099,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>Genesis, Voyager, BlockFi debtors - context only</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="8" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="8" t="n"/>
     </row>
     <row r="16" ht="92" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -1164,7 +2125,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Investment Banking - FINTECH &amp; WEALTH group (within FIG). Technology group adjacent. Full ECM platform in-house.</t>
+          <t>The only firm combining three crypto M&amp;A sell-sides, the largest associate class of the group, a named fintech group, and a CBS alum leading that exact team.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1189,15 +2150,10 @@
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>FTX creditors committee - context only</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
           <t>John Erwin - MD, FinTech &amp; Wealth Investment Banking, CBS MBA '06</t>
         </is>
       </c>
-      <c r="L16" s="8" t="n"/>
+      <c r="K16" s="8" t="n"/>
     </row>
     <row r="17" ht="92" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -1245,13 +2201,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="n"/>
-      <c r="L17" s="8" t="n"/>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="8" t="n"/>
     </row>
     <row r="18" ht="92" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -1276,7 +2227,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Generalist advisory - no formal industry groups; industry-agnostic staffing.</t>
+          <t>ZERO crypto M&amp;A credits. Industry-agnostic staffing (no formal groups) and the smallest associate class in the market.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1299,13 +2250,8 @@
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>Celsius Ch.11 debtors (~$20.1M fee allocation) - context only</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="n"/>
-      <c r="L18" s="8" t="n"/>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="8" t="n"/>
     </row>
     <row r="19" ht="92" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -1330,7 +2276,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Single Advisory platform (M&amp;A and restructuring are not separately branded).</t>
+          <t>ZERO crypto M&amp;A credits — no crypto M&amp;A franchise to point at. FIG coverage exists but the crypto work is not M&amp;A.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1353,13 +2299,8 @@
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>FTX debtors (ran the LedgerX and FTX Europe sales); Celsius creditors - context only</t>
-        </is>
-      </c>
-      <c r="K19" s="6" t="n"/>
-      <c r="L19" s="8" t="n"/>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="8" t="n"/>
     </row>
     <row r="20" ht="92" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -1384,7 +2325,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>CORPORATE FINANCE (M&amp;A) - has a real FinTech group. Financial Restructuring is the separate arm where the crypto work sat.</t>
+          <t>Apply to CORPORATE FINANCE — that is the M&amp;A division and it houses the FinTech group. HL ranks #1 globally in M&amp;A by deal COUNT and is mid-market focused, which matches where most crypto deals actually clear. Zero crypto M&amp;A credits, so this is a fintech pitch, not a crypto one.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1407,13 +2348,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>Genesis creditors - context only</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="n"/>
-      <c r="L20" s="8" t="n"/>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="8" t="n"/>
     </row>
     <row r="21" ht="92" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -1461,13 +2397,8 @@
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="n"/>
-      <c r="L21" s="8" t="n"/>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="8" t="n"/>
     </row>
     <row r="22" ht="92" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -1515,13 +2446,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K22" s="6" t="n"/>
-      <c r="L22" s="8" t="n"/>
+      <c r="J22" s="6" t="n"/>
+      <c r="K22" s="8" t="n"/>
     </row>
     <row r="23" ht="92" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -1571,15 +2497,10 @@
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>None - no restructuring practice</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
           <t>Mike Pascucci - Managing Director, CBS MBA '12</t>
         </is>
       </c>
-      <c r="L23" s="8" t="n"/>
+      <c r="K23" s="8" t="n"/>
     </row>
     <row r="24" ht="92" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -1627,13 +2548,8 @@
           <t>Twenty One Capital (FA + placement, Apr 2025; NYSE: XXI Dec 2025 - the Tether/SoftBank vehicle); Securitize $1.25B pre-money (buy-side FA for CEPT, Oct 2025); bitcoin financing book</t>
         </is>
       </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="n"/>
-      <c r="L24" s="8" t="n"/>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="8" t="n"/>
     </row>
     <row r="25" ht="92" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -1683,15 +2599,10 @@
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
           <t>Christian J. Lopez - MD, HEAD of Blockchain &amp; Digital Assets, CBS MBA. Also Rahul Jasuja - MD, Energy &amp; Energy Transition IB, CBS MBA; Pawel Skonieczka - MD, CBS MBA '13</t>
         </is>
       </c>
-      <c r="L25" s="8" t="n"/>
+      <c r="K25" s="8" t="n"/>
     </row>
     <row r="26" ht="92" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -1739,13 +2650,8 @@
           <t>FIG ECM is a core KBW franchise - the natural home for crypto-bank and stablecoin-issuer issuance. Verify specific roles.</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="8" t="n"/>
+      <c r="J26" s="6" t="n"/>
+      <c r="K26" s="8" t="n"/>
     </row>
     <row r="27" ht="92" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
@@ -1795,15 +2701,10 @@
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K27" s="6" t="inlineStr">
-        <is>
           <t>Jerry von Dohlen - Founder &amp; Partner, CBS MBA '96 (+ Columbia Engineering BS); James Denton - Partner, CBS MBA '85</t>
         </is>
       </c>
-      <c r="L27" s="8" t="n"/>
+      <c r="K27" s="8" t="n"/>
     </row>
     <row r="28" ht="92" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
@@ -1851,13 +2752,8 @@
           <t>Galaxy Global Markets runs financing/structured products - adjacent to ECM but not underwriting.</t>
         </is>
       </c>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="8" t="n"/>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="8" t="n"/>
     </row>
     <row r="29" ht="92" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1905,13 +2801,8 @@
           <t>No ECM practice.</t>
         </is>
       </c>
-      <c r="J29" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="8" t="n"/>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="8" t="n"/>
     </row>
     <row r="30" ht="92" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
@@ -1961,15 +2852,10 @@
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="inlineStr">
-        <is>
           <t>Collin Finnerty - MD, Blockchain &amp; Digital Infrastructure Investment Banking, CBS MBA '20</t>
         </is>
       </c>
-      <c r="L30" s="8" t="n"/>
+      <c r="K30" s="8" t="n"/>
     </row>
     <row r="31" ht="92" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -2019,15 +2905,10 @@
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K31" s="6" t="inlineStr">
-        <is>
           <t>Rob Brown - CEO, CBS MBA; Scott Twibell - MD Global Co-Head Technology; Steve Carre, Brian Goodwin, Mark Karasik, Mark Y. (MDs); Dave Reese (Director); Cole Ahnell (Associate, CBS '23); Mike Zhang (Analyst, CBS MS '24)</t>
         </is>
       </c>
-      <c r="L31" s="8" t="n"/>
+      <c r="K31" s="8" t="n"/>
     </row>
     <row r="32" ht="92" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
@@ -2075,13 +2956,8 @@
           <t>Research-driven capital markets; verify crypto issuance roles.</t>
         </is>
       </c>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="8" t="n"/>
+      <c r="J32" s="6" t="n"/>
+      <c r="K32" s="8" t="n"/>
     </row>
     <row r="33" ht="92" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
@@ -2129,13 +3005,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J33" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="8" t="n"/>
+      <c r="J33" s="6" t="n"/>
+      <c r="K33" s="8" t="n"/>
     </row>
     <row r="34" ht="92" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
@@ -2183,13 +3054,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J34" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="8" t="n"/>
+      <c r="J34" s="6" t="n"/>
+      <c r="K34" s="8" t="n"/>
     </row>
     <row r="35" ht="92" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
@@ -2237,13 +3103,8 @@
           <t>No disclosed crypto ECM.</t>
         </is>
       </c>
-      <c r="J35" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K35" s="6" t="n"/>
-      <c r="L35" s="8" t="n"/>
+      <c r="J35" s="6" t="n"/>
+      <c r="K35" s="8" t="n"/>
     </row>
     <row r="36" ht="92" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -2291,13 +3152,8 @@
           <t>Digital assets capital markets is the stated franchise - verify specific issuance roles.</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="8" t="n"/>
+      <c r="J36" s="6" t="n"/>
+      <c r="K36" s="8" t="n"/>
     </row>
     <row r="37" ht="92" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -2345,13 +3201,8 @@
           <t>Research-led digital assets capital markets - verify issuance roles.</t>
         </is>
       </c>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K37" s="6" t="n"/>
-      <c r="L37" s="8" t="n"/>
+      <c r="J37" s="6" t="n"/>
+      <c r="K37" s="8" t="n"/>
     </row>
     <row r="38" ht="92" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
@@ -2399,13 +3250,8 @@
           <t>None disclosed</t>
         </is>
       </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K38" s="6" t="n"/>
-      <c r="L38" s="8" t="n"/>
+      <c r="J38" s="6" t="n"/>
+      <c r="K38" s="8" t="n"/>
     </row>
     <row r="39" ht="92" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
@@ -2455,15 +3301,10 @@
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
           <t>Phillip Kim - Managing Director, CBS MBA '05; Joe Josephson - Partner (CBS '98)</t>
         </is>
       </c>
-      <c r="L39" s="8" t="n"/>
+      <c r="K39" s="8" t="n"/>
     </row>
     <row r="40" ht="92" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
@@ -2511,13 +3352,8 @@
           <t>Major FIG ECM franchise - context only</t>
         </is>
       </c>
-      <c r="J40" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="n"/>
-      <c r="L40" s="8" t="n"/>
+      <c r="J40" s="6" t="n"/>
+      <c r="K40" s="8" t="n"/>
     </row>
     <row r="41" ht="92" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -2565,13 +3401,8 @@
           <t>Mid-market ECM - context only</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K41" s="6" t="n"/>
-      <c r="L41" s="8" t="n"/>
+      <c r="J41" s="6" t="n"/>
+      <c r="K41" s="8" t="n"/>
     </row>
     <row r="42" ht="92" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2619,13 +3450,8 @@
           <t>Mid-market ECM - context only</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K42" s="6" t="n"/>
-      <c r="L42" s="8" t="n"/>
+      <c r="J42" s="6" t="n"/>
+      <c r="K42" s="8" t="n"/>
     </row>
     <row r="43" ht="92" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -2673,13 +3499,8 @@
           <t>Limited</t>
         </is>
       </c>
-      <c r="J43" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K43" s="6" t="n"/>
-      <c r="L43" s="8" t="n"/>
+      <c r="J43" s="6" t="n"/>
+      <c r="K43" s="8" t="n"/>
     </row>
     <row r="44" ht="92" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
@@ -2727,15 +3548,9 @@
           <t>No ECM - pure advisory</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr">
-        <is>
-          <t>None in crypto</t>
-        </is>
-      </c>
-      <c r="K44" s="6" t="n"/>
-      <c r="L44" s="8" t="n"/>
-    </row>
-    <row r="45"/>
+      <c r="J44" s="6" t="n"/>
+      <c r="K44" s="8" t="n"/>
+    </row>
     <row r="46" ht="100" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
@@ -2744,7 +3559,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:L44"/>
+  <autoFilter ref="A5:K44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix restructuring scrub to correct column after OCR insert
Rewrites had landed one column left of the notes field. Bank Profiles
is now clean of restructuring language except the deliberate PJT
Strategic-Advisory-not-RSSG guardrail.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WXzZsq4Qrn4tV9mBn34Mo
</commit_message>
<xml_diff>
--- a/IB_Target_Profiles.xlsx
+++ b/IB_Target_Profiles.xlsx
@@ -1531,7 +1531,7 @@
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>M&amp;A-FIRST view: target-group precision for the crypto/fintech M&amp;A lane  |  ECM and restructuring credits shown separately as CONTEXT ONLY  |  CBS Class of 2028, summer 2027 associate cycle</t>
+          <t>M&amp;A-FIRST view: target-group precision for the crypto/fintech M&amp;A lane  |  ECM credits shown separately as CONTEXT ONLY  |  CBS Class of 2028, summer 2027 associate cycle</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>CRITICAL: RSSG (Restructuring &amp; Special Situations Group) is a separate, MBA-heavy track and is where the Core Scientific Ch.11 sat - the tracks split early. Park Hill (fund placement) is a third arm. All the Payward M&amp;A work is Strategic Advisory. Say 'strategic advisory' in every conversation.</t>
+          <t>CRITICAL: PJT has four arms — Strategic Advisory (M&amp;A, your target), RSSG, Park Hill (fund placement) and Camberview (shareholder advisory). All the Payward M&amp;A work is Strategic Advisory. Say 'strategic advisory' in every conversation so you are not routed elsewhere.</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Its crypto reputation is 60% restructuring (Voyager, Genesis, BlockFi debtors). If you have ruled out Rx, only two of its five credits are relevant - and staffing can cross between M&amp;A and R&amp;R.</t>
+          <t>Generalist FIG / M&amp;A coverage with two crypto M&amp;A credits. Associate staffing is broad across the platform. No named fintech group and no alumni door.</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Only firm combining three crypto M&amp;A sell-sides, real ECM, the largest associate class of the group, and a CBS alum leading the exact coverage group.</t>
+          <t>The only firm combining three crypto M&amp;A sell-sides, the largest associate class of the group, a named fintech group, and a CBS alum leading that exact team.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -2232,7 +2232,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>ZERO crypto M&amp;A credits. Its only crypto work is the Celsius Ch.11 debtor role. Smallest class in the market.</t>
+          <t>ZERO crypto M&amp;A credits. Industry-agnostic staffing (no formal groups) and the smallest associate class in the market.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>ZERO crypto M&amp;A credits. Both crypto engagements are restructuring - FTX debtors and Celsius creditors. Its crypto reputation is entirely estates.</t>
+          <t>ZERO crypto M&amp;A credits — no crypto M&amp;A franchise to point at. FIG coverage exists but the crypto work was never M&amp;A.</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>ZERO crypto M&amp;A credits; the Genesis role was creditor-side Rx. The Corporate Finance FinTech group is legitimate for fintech M&amp;A - but that is a fintech pitch, not a crypto one.</t>
+          <t>Apply to CORPORATE FINANCE — that is the M&amp;A division and it houses the FinTech group. HL ranks #1 globally in M&amp;A by deal COUNT and is mid-market focused, which matches where most crypto deals actually clear. Zero crypto M&amp;A credits, so this is a fintech pitch, not a crypto one.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>The single purest fintech M&amp;A franchise on this list: 100% fintech, zero restructuring. Hires associates DIRECTLY via Greenhouse (no OCR), so it does not compete with your Sept-Jan calendar. Culture is famously demanding - diligence with former juniors before committing.</t>
+          <t>The single purest fintech M&amp;A franchise on this list: 100% fintech, no other business lines diluting the work. Hires associates DIRECTLY via Greenhouse (no OCR), so it does not compete with your Sept–Jan calendar. Culture is famously demanding — diligence with former juniors before committing.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3551,10 +3551,11 @@
       <c r="J44" s="6" t="n"/>
       <c r="K44" s="8" t="n"/>
     </row>
+    <row r="45"/>
     <row r="46" ht="100" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>Deal mandates are advisor attributions verified from press releases, law-firm and bank announcements, SEC filings and Architect Partners M&amp;A alerts through Aug 21, 2026 — 'Not disclosed' on a transaction means no public attribution was found, not that no advisor was engaged, so several firms will have more credits than are listed. GROUP AND DEPARTMENT NAMES ARE FROM GENERAL KNOWLEDGE (Jan 2026 horizon) and banks rename and reorganize coverage groups constantly — confirm the exact group name on the firm's site or in your first conversation before using it. Items marked VERIFY are explicitly unconfirmed. ECM entries are thinner than M&amp;A across the board because underwriting syndicates are less consistently disclosed than advisory mandates; confirm bookrunner roles on the crypto IPO wave (Circle CRCL Jun 2025, Gemini GEMI Sep 2025, Bullish) directly from the prospectuses. Restructuring column is included so you can see which firms' crypto reputations rest entirely on estates work.</t>
+          <t>Deal mandates are advisor attributions verified from press releases, law-firm and bank announcements, SEC filings and Architect Partners M&amp;A alerts through Aug 21, 2026 — 'None disclosed' means no public attribution was found, not that no adviser was engaged, so several firms will have more credits than are listed. GROUP AND DEPARTMENT NAMES ARE FROM GENERAL KNOWLEDGE (Jan 2026 horizon) and banks rename coverage groups constantly — confirm the exact group name on the firm's site or in your first conversation before using it. OCR status reflects general MBA-recruiting patterns plus your Aug 2026 tracker; CBS's live roster is on the CMC portal — reconcile it in week one. Items marked VERIFY are explicitly unconfirmed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct FT Partners entry route after direct research
Three independent searches: FT Partners' structured summer programme is
UNDERGRADUATE (college juniors, SAT/ACT required, posts as Summer
Analyst). Associate roles are experienced-hire laterals requiring 2+
years full-time IB in M&A sell-side advisory plus FINRA Series 63/79.
No evidence of an MBA summer associate programme. Re-scoped as a
full-time-2028/lateral target; George plausibly clears the lateral bar
via Brasilpar. One ambiguous source warrants a direct check with
recruiting@ftpartners.com.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WXzZsq4Qrn4tV9mBn34Mo
</commit_message>
<xml_diff>
--- a/IB_Target_Profiles.xlsx
+++ b/IB_Target_Profiles.xlsx
@@ -596,17 +596,17 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>NO — direct application via Greenhouse</t>
+          <t>NO — and likely NO MBA summer associate programme at all (researched Aug 2026)</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Investment Banking associate programme; ask for the BLOCKCHAIN / DIGITAL ASSETS vertical. No departments — the firm organises in deal teams.</t>
+          <t>Investment Banking, BLOCKCHAIN / DIGITAL ASSETS vertical — but note the entry route: their structured summer programme is an UNDERGRAD Summer ANALYST programme (college juniors, SAT/ACT required). Associate roles are EXPERIENCED-HIRE laterals: 2+ yrs full-time IB in M&amp;A sell-side advisory, FINRA Series 63 + 79. Apply direct via Greenhouse / recruiting@ftpartners.com.</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>YOUR PICK. The purest fit on the list: four crypto M&amp;A sell-sides, 100% fintech, no other business lines diluting the work. Applies outside OCR so it costs you nothing in Sept–Jan. Diligence the culture with former juniors before committing.</t>
+          <t>YOUR PICK, but re-scope it: this is a FULL-TIME 2028 / lateral target, not a summer-2027 seat. The good news — you plausibly clear their lateral bar already: Brasilpar was ~2 yrs as an M&amp;A analyst on live buy- and sell-side mandates, which is exactly what they ask for. Series 63/79 are normally obtained post-offer under sponsorship. Most MBAs cannot make that argument; you can. ACTION: email recruiting@ftpartners.com and ask directly whether an MBA summer associate programme exists for 2027 — one ambiguous source says summer interns sit as 'Analyst or Associate'.</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
@@ -1485,6 +1485,7 @@
       </c>
       <c r="H30" s="8" t="n"/>
     </row>
+    <row r="31"/>
     <row r="32" ht="74" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
@@ -2462,7 +2463,7 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>NO — direct via Greenhouse</t>
+          <t>NO — undergrad Summer Analyst programme only; associates are experienced-hire laterals</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2477,7 +2478,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>The single purest fintech M&amp;A franchise on this list: 100% fintech, no other business lines diluting the work. Hires associates DIRECTLY via Greenhouse (no OCR), so it does not compete with your Sept–Jan calendar. Culture is famously demanding — diligence with former juniors before committing.</t>
+          <t>The purest fintech M&amp;A franchise on this list: 100% fintech, no other business lines diluting the work. ENTRY ROUTE (researched Aug 2026): the structured summer programme is UNDERGRADUATE (college juniors, GPA 3.5+, SAT/ACT score report required) and posts as 'Summer Analyst'. Associate roles are experienced hires — 2+ years full-time IB in M&amp;A sell-side advisory plus FINRA Series 63 and 79. Realistic path is full-time/lateral post-MBA, pitching prior M&amp;A analyst experience. Verify directly: recruiting@ftpartners.com. Culture is famously demanding — diligence with former juniors.</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Correct Cantor Fitzgerald after research; promote 22 -> 11
Cantor runs a full-service IB (ECM, DCM, M&A, restructuring) under Sage
Kelly as Co-CEO and Global Head of IB, with Digital Assets as a NAMED
coverage sector and a fast-growing Technology group covering fintech.
~46 M&A deals vs 84 funding rounds. Prior 'mostly capital markets, low
priority' framing at rank 22 was too harsh: two named groups match a
fintech/crypto mandate.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WXzZsq4Qrn4tV9mBn34Mo
</commit_message>
<xml_diff>
--- a/IB_Target_Profiles.xlsx
+++ b/IB_Target_Profiles.xlsx
@@ -951,27 +951,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Houlihan Lokey</t>
+          <t>Cantor Fitzgerald</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>YES — OCR</t>
+          <t>NO — posts roles; less structured MBA path</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>CORPORATE FINANCE — FinTech group. (Corporate Finance is the M&amp;A division.)</t>
+          <t>TWO qualifying entry points: (a) DIGITAL ASSETS — a named sector coverage team; or (b) TECHNOLOGY group, which covers fintech and is the fastest-growing team on the platform (nine senior hires). Cantor Equity Partners (CEP/CEPT) are the affiliated SPAC vehicles — separate. Bitcoin financing desk separate again.</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>#1 globally in M&amp;A by deal count and mid-market focused, which matches where most crypto deals actually clear. Zero crypto credits — a fintech pitch only.</t>
+          <t>CORRECTED Aug 2026 after direct research: Cantor runs a full-service IB — ECM, DCM, M&amp;A and restructuring under Sage Kelly, Co-CEO and Global Head of IB — and Digital Assets is a NAMED coverage sector. Deal mix ~46 M&amp;A to 84 funding rounds, so capital-markets weighted, but the M&amp;A practice is real. Crypto flow to date is DAT/de-SPAC heavy. Two named groups matching your mandate is more than most banks offer.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>None in crypto; high-volume mid-market fintech M&amp;A</t>
+          <t>Semler Scientific ~$1.4B (buy-side FA to Strive, Sep 2025). Digital Assets flow to date DAT/de-SPAC weighted: Twenty One Capital (Apr 2025); Securitize $1.25B (Oct 2025).</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -987,27 +987,27 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>LionTree</t>
+          <t>Houlihan Lokey</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>NO — relationship-driven</t>
+          <t>YES — OCR</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Generalist merchant bank, TMT and media focus. No fintech or crypto group — approach the firm, not a desk.</t>
+          <t>CORPORATE FINANCE — FinTech group. (Corporate Finance is the M&amp;A division.)</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Ran the exclusive Semler sell-side, the first DAT stock-for-stock merger. Real digital-asset appetite but a very small intake.</t>
+          <t>#1 globally in M&amp;A by deal count and mid-market focused, which matches where most crypto deals actually clear. Zero crypto credits — a fintech pitch only.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Semler Scientific ~$1.4B (EXCL. sell vs Strive, Sep 2025); Equiniti $4.2B (sell syndicate, May 2026)</t>
+          <t>None in crypto; high-volume mid-market fintech M&amp;A</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1023,27 +1023,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Moelis</t>
+          <t>LionTree</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>YES — OCR</t>
+          <t>NO — relationship-driven</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Investment Banking — FIG (generalist M&amp;A coverage).</t>
+          <t>Generalist merchant bank, TMT and media focus. No fintech or crypto group — approach the firm, not a desk.</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Two crypto M&amp;A credits and full OCR access. Solid, not differentiated — no named fintech group and no alumni door.</t>
+          <t>Ran the exclusive Semler sell-side, the first DAT stock-for-stock merger. Real digital-asset appetite but a very small intake.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Stronghold Digital $125M (buy, Bitfarms, Aug 2024); Core Scientific $9B (co-sell with PJT, Jul 2025)</t>
+          <t>Semler Scientific ~$1.4B (EXCL. sell vs Strive, Sep 2025); Equiniti $4.2B (sell syndicate, May 2026)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>JPMorgan</t>
+          <t>Moelis</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -1069,17 +1069,17 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Investment Banking — FIG, FINANCIAL TECHNOLOGY coverage. (Kinexys is a product unit, not IB — do not target it.)</t>
+          <t>Investment Banking — FIG (generalist M&amp;A coverage).</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Dedicated fintech coverage and a huge platform. Note the Adecoagro mandate came from LatAm/agri coverage, not fintech — so the crypto flow into the fintech team is thinner than the credit count suggests.</t>
+          <t>Two crypto M&amp;A credits and full OCR access. Solid, not differentiated — no named fintech group and no alumni door.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Adecoagro ~$615.5M (excl. sell vs Tether, Mar 2025); WonderFi C$250M (buy, Robinhood, May 2025)</t>
+          <t>Stronghold Digital $125M (buy, Bitfarms, Aug 2024); Core Scientific $9B (co-sell with PJT, Jul 2025)</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1095,32 +1095,32 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Clear Street</t>
+          <t>JPMorgan</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>VERIFY — growing platform</t>
+          <t>YES — OCR</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Investment Banking — BLOCKCHAIN &amp; DIGITAL INFRASTRUCTURE group.</t>
+          <t>Investment Banking — FIG, FINANCIAL TECHNOLOGY coverage. (Kinexys is a product unit, not IB — do not target it.)</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>A crypto-native IB group run by a CBS alum inside a prime broker — directly adjacent to your COR PRIME operating background. No lead M&amp;A credit yet.</t>
+          <t>Dedicated fintech coverage and a huge platform. Note the Adecoagro mandate came from LatAm/agri coverage, not fintech — so the crypto flow into the fintech team is thinner than the credit count suggests.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>None as lead adviser; co-placement on ProCap ~$1B (Jun 2025)</t>
+          <t>Adecoagro ~$615.5M (excl. sell vs Tether, Mar 2025); WonderFi C$250M (buy, Robinhood, May 2025)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Collin Finnerty — MD, Blockchain &amp; Digital Infrastructure IB, CBS MBA '20</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H20" s="8" t="n"/>
@@ -1131,32 +1131,32 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Piper Sandler</t>
+          <t>Clear Street</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>VERIFY — runs MBA recruiting; confirm CBS</t>
+          <t>VERIFY — growing platform</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Financial Services Group — FinTech coverage (built on the absorbed Sandler O'Neill FIG franchise).</t>
+          <t>Investment Banking — BLOCKCHAIN &amp; DIGITAL INFRASTRUCTURE group.</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>One of the deepest FIG franchises on the street and the biggest gap in your original list. No crypto credit — a fintech pitch.</t>
+          <t>A crypto-native IB group run by a CBS alum inside a prime broker — directly adjacent to your COR PRIME operating background. No lead M&amp;A credit yet.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>None surfaced in crypto; high-volume bank, specialty finance and payments M&amp;A</t>
+          <t>None as lead adviser; co-placement on ProCap ~$1B (Jun 2025)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Collin Finnerty — MD, Blockchain &amp; Digital Infrastructure IB, CBS MBA '20</t>
         </is>
       </c>
       <c r="H21" s="8" t="n"/>
@@ -1167,27 +1167,27 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Lazard</t>
+          <t>Piper Sandler</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>YES — OCR</t>
+          <t>VERIFY — runs MBA recruiting; confirm CBS</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Financial Advisory — FIG.</t>
+          <t>Financial Services Group — FinTech coverage (built on the absorbed Sandler O'Neill FIG franchise).</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>One credit, and it came through Power &amp; Energy Infrastructure (FTAI was a power asset), not a digital-assets franchise. Portfolio filler.</t>
+          <t>One of the deepest FIG franchises on the street and the biggest gap in your original list. No crypto credit — a fintech pitch.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Long Ridge $1.5B (co-sell for FTAI, Apr 2026)</t>
+          <t>None surfaced in crypto; high-volume bank, specialty finance and payments M&amp;A</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -1203,32 +1203,32 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Union Square Advisors</t>
+          <t>Lazard</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>VERIFY — small, likely direct</t>
+          <t>YES — OCR</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Technology M&amp;A — FINTECH vertical.</t>
+          <t>Financial Advisory — FIG.</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Pure tech M&amp;A boutique with a CBS MD. No crypto credit — fintech framing only.</t>
+          <t>One credit, and it came through Power &amp; Energy Infrastructure (FTAI was a power asset), not a digital-assets franchise. Portfolio filler.</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>None disclosed in crypto</t>
+          <t>Long Ridge $1.5B (co-sell for FTAI, Apr 2026)</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Phillip Kim — Managing Director, CBS MBA '05</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H23" s="8" t="n"/>
@@ -1239,32 +1239,32 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>William Blair</t>
+          <t>Union Square Advisors</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>VERIFY — has MBA summer associate programme; confirm CBS</t>
+          <t>VERIFY — small, likely direct</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Technology &amp; Services — FINTECH / PAYMENTS coverage.</t>
+          <t>Technology M&amp;A — FINTECH vertical.</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Active upper-middle-market fintech and payments M&amp;A. No crypto credit.</t>
+          <t>Pure tech M&amp;A boutique with a CBS MD. No crypto credit — fintech framing only.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>None surfaced in crypto; recurring payments and fintech M&amp;A</t>
+          <t>None disclosed in crypto</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Phillip Kim — Managing Director, CBS MBA '05</t>
         </is>
       </c>
       <c r="H24" s="8" t="n"/>
@@ -1275,32 +1275,32 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Lincoln International</t>
+          <t>William Blair</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>VERIFY — has hired CBS MBA associates</t>
+          <t>VERIFY — has MBA summer associate programme; confirm CBS</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Technology group (fintech sits within Technology / Business Services).</t>
+          <t>Technology &amp; Services — FINTECH / PAYMENTS coverage.</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Nine CBS people including the CEO — the densest alumni cluster of any bank here — but one crypto credit and a mid-market generalist mandate.</t>
+          <t>Active upper-middle-market fintech and payments M&amp;A. No crypto credit.</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>GRIID Infrastructure $155M (sell FA + fairness opinion, CleanSpark, Jun 2024)</t>
+          <t>None surfaced in crypto; recurring payments and fintech M&amp;A</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Rob Brown — CEO, CBS MBA; Cole Ahnell — Associate, CBS '23; plus 7 more</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H25" s="8" t="n"/>
@@ -1311,32 +1311,32 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Arma Partners</t>
+          <t>Lincoln International</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>NO — European, no US OCR</t>
+          <t>VERIFY — has hired CBS MBA associates</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>FinTech sector team (London).</t>
+          <t>Technology group (fintech sits within Technology / Business Services).</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Europe's leading independent digital-economy adviser and a natural fit for your London network. No crypto credit surfaced.</t>
+          <t>Nine CBS people including the CEO — the densest alumni cluster of any bank here — but one crypto credit and a mid-market generalist mandate.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>None surfaced in crypto; heavy European fintech and software M&amp;A</t>
+          <t>GRIID Infrastructure $155M (sell FA + fairness opinion, CleanSpark, Jun 2024)</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Rob Brown — CEO, CBS MBA; Cole Ahnell — Associate, CBS '23; plus 7 more</t>
         </is>
       </c>
       <c r="H26" s="8" t="n"/>
@@ -1347,27 +1347,27 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Cantor Fitzgerald</t>
+          <t>Arma Partners</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>NO — posts roles, unstructured</t>
+          <t>NO — European, no US OCR</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>DIGITAL ASSETS group within Cantor Fitzgerald &amp; Co. investment banking.</t>
+          <t>FinTech sector team (London).</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Named digital-assets group, but the franchise is capital markets and DAT vehicles — only one M&amp;A credit. Low priority on an M&amp;A-only mandate.</t>
+          <t>Europe's leading independent digital-economy adviser and a natural fit for your London network. No crypto credit surfaced.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Semler Scientific ~$1.4B (buy-side FA to Strive, Sep 2025)</t>
+          <t>None surfaced in crypto; heavy European fintech and software M&amp;A</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -2526,12 +2526,12 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>DIGITAL ASSETS GROUP within Cantor Fitzgerald &amp; Co. investment banking. Cantor Equity Partners (CEP, CEPT) are the affiliated SPAC sponsor vehicles. Bitcoin financing desk is separate again.</t>
+          <t>TWO options: DIGITAL ASSETS (named sector coverage team) or the TECHNOLOGY group (covers fintech; fastest-growing team on the platform). Cantor Equity Partners (CEP/CEPT) are the affiliated SPAC sponsor vehicles — separate. Bitcoin financing desk separate again.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>The deepest crypto ECM franchise in the market - if ECM genuinely interests you this is the highest-conviction name on the list. Be clear which arm you are targeting: advisory vs the SPAC sponsor vehicles vs bitcoin financing. Risk: DAT-lane concentration and the post-2025 derating of treasury companies.</t>
+          <t>CORRECTED Aug 2026 after direct research: full-service IB — ECM, DCM, M&amp;A and restructuring under Sage Kelly, Co-CEO and Global Head of Investment Banking. Digital Assets is a NAMED coverage sector. ~46 M&amp;A deals vs 84 funding rounds — capital-markets weighted but M&amp;A is substantial. Crypto flow to date is DAT/de-SPAC heavy.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">

</xml_diff>